<commit_message>
Update Artesian valuation model
</commit_message>
<xml_diff>
--- a/public/research/initial-screenings/Initial Screening (Under 1B MC, Over $0 NI).xlsx
+++ b/public/research/initial-screenings/Initial Screening (Under 1B MC, Over $0 NI).xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1581" uniqueCount="744">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1587" uniqueCount="744">
   <si>
     <t>Entity Name</t>
   </si>
@@ -2177,24 +2177,27 @@
     <t>Valuation Template</t>
   </si>
   <si>
+    <t>Technology</t>
+  </si>
+  <si>
+    <t>N/M</t>
+  </si>
+  <si>
     <t>Declining / Cigar-Butt / Runoff Cash Flow Template</t>
   </si>
   <si>
+    <t>Consumer Goods</t>
+  </si>
+  <si>
     <t>Fail</t>
   </si>
   <si>
     <t>LINK</t>
   </si>
   <si>
-    <t>Technology</t>
-  </si>
-  <si>
     <t>Subscription / Software / Intangible-Asset Business Template</t>
   </si>
   <si>
-    <t>Consumer Goods</t>
-  </si>
-  <si>
     <t>Cyclical / Normalized Earnings Template</t>
   </si>
   <si>
@@ -2220,9 +2223,6 @@
   </si>
   <si>
     <t>Watchlist</t>
-  </si>
-  <si>
-    <t>N/M</t>
   </si>
   <si>
     <t>Energy</t>
@@ -2355,13 +2355,13 @@
     <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" vertical="center"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
   </cellXfs>
@@ -20013,7 +20013,7 @@
     <col customWidth="1" min="1" max="1" width="46.29"/>
     <col customWidth="1" min="2" max="2" width="12.86"/>
     <col customWidth="1" min="3" max="3" width="18.29"/>
-    <col customWidth="1" min="4" max="4" width="12.14"/>
+    <col customWidth="1" min="4" max="4" width="15.71"/>
     <col customWidth="1" min="5" max="5" width="11.43"/>
     <col customWidth="1" min="6" max="6" width="8.43"/>
     <col customWidth="1" min="7" max="7" width="51.71"/>
@@ -20067,8 +20067,14 @@
         <f>IFERROR(__xludf.DUMMYFUNCTION("FILTER('Phase 1'!A2:A1000,'Phase 1'!K2:K1000=""PASS"")"),"AirJoule Technologies Corporation (NASDAQCM:AIRJ)")</f>
         <v>AirJoule Technologies Corporation (NASDAQCM:AIRJ)</v>
       </c>
+      <c r="D2" s="5" t="s">
+        <v>719</v>
+      </c>
+      <c r="F2" s="13" t="s">
+        <v>720</v>
+      </c>
       <c r="G2" s="5" t="s">
-        <v>719</v>
+        <v>721</v>
       </c>
     </row>
     <row r="3">
@@ -20076,8 +20082,14 @@
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Beazer Homes USA, Inc. (NYSE:BZH)")</f>
         <v>Beazer Homes USA, Inc. (NYSE:BZH)</v>
       </c>
+      <c r="D3" s="5" t="s">
+        <v>722</v>
+      </c>
+      <c r="F3" s="13" t="s">
+        <v>720</v>
+      </c>
       <c r="G3" s="5" t="s">
-        <v>719</v>
+        <v>721</v>
       </c>
     </row>
     <row r="4">
@@ -20085,8 +20097,14 @@
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Calavo Growers, Inc. (NASDAQGS:CVGW)")</f>
         <v>Calavo Growers, Inc. (NASDAQGS:CVGW)</v>
       </c>
+      <c r="D4" s="5" t="s">
+        <v>722</v>
+      </c>
+      <c r="F4" s="13">
+        <v>29.0</v>
+      </c>
       <c r="G4" s="5" t="s">
-        <v>719</v>
+        <v>721</v>
       </c>
     </row>
     <row r="5">
@@ -20094,9 +20112,3000 @@
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Coffee Holding Co., Inc. (NASDAQCM:JVA)")</f>
         <v>Coffee Holding Co., Inc. (NASDAQCM:JVA)</v>
       </c>
+      <c r="D5" s="5" t="s">
+        <v>722</v>
+      </c>
+      <c r="F5" s="13">
+        <v>13.1</v>
+      </c>
       <c r="G5" s="5" t="s">
-        <v>719</v>
-      </c>
+        <v>721</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="F6" s="7"/>
+    </row>
+    <row r="7">
+      <c r="F7" s="7"/>
+    </row>
+    <row r="8">
+      <c r="F8" s="7"/>
+    </row>
+    <row r="9">
+      <c r="F9" s="7"/>
+    </row>
+    <row r="10">
+      <c r="F10" s="7"/>
+    </row>
+    <row r="11">
+      <c r="F11" s="7"/>
+    </row>
+    <row r="12">
+      <c r="F12" s="7"/>
+    </row>
+    <row r="13">
+      <c r="F13" s="7"/>
+    </row>
+    <row r="14">
+      <c r="F14" s="7"/>
+    </row>
+    <row r="15">
+      <c r="F15" s="7"/>
+    </row>
+    <row r="16">
+      <c r="F16" s="7"/>
+    </row>
+    <row r="17">
+      <c r="F17" s="7"/>
+    </row>
+    <row r="18">
+      <c r="F18" s="7"/>
+    </row>
+    <row r="19">
+      <c r="F19" s="7"/>
+    </row>
+    <row r="20">
+      <c r="F20" s="7"/>
+    </row>
+    <row r="21">
+      <c r="F21" s="7"/>
+    </row>
+    <row r="22">
+      <c r="F22" s="7"/>
+    </row>
+    <row r="23">
+      <c r="F23" s="7"/>
+    </row>
+    <row r="24">
+      <c r="F24" s="7"/>
+    </row>
+    <row r="25">
+      <c r="F25" s="7"/>
+    </row>
+    <row r="26">
+      <c r="F26" s="7"/>
+    </row>
+    <row r="27">
+      <c r="F27" s="7"/>
+    </row>
+    <row r="28">
+      <c r="F28" s="7"/>
+    </row>
+    <row r="29">
+      <c r="F29" s="7"/>
+    </row>
+    <row r="30">
+      <c r="F30" s="7"/>
+    </row>
+    <row r="31">
+      <c r="F31" s="7"/>
+    </row>
+    <row r="32">
+      <c r="F32" s="7"/>
+    </row>
+    <row r="33">
+      <c r="F33" s="7"/>
+    </row>
+    <row r="34">
+      <c r="F34" s="7"/>
+    </row>
+    <row r="35">
+      <c r="F35" s="7"/>
+    </row>
+    <row r="36">
+      <c r="F36" s="7"/>
+    </row>
+    <row r="37">
+      <c r="F37" s="7"/>
+    </row>
+    <row r="38">
+      <c r="F38" s="7"/>
+    </row>
+    <row r="39">
+      <c r="F39" s="7"/>
+    </row>
+    <row r="40">
+      <c r="F40" s="7"/>
+    </row>
+    <row r="41">
+      <c r="F41" s="7"/>
+    </row>
+    <row r="42">
+      <c r="F42" s="7"/>
+    </row>
+    <row r="43">
+      <c r="F43" s="7"/>
+    </row>
+    <row r="44">
+      <c r="F44" s="7"/>
+    </row>
+    <row r="45">
+      <c r="F45" s="7"/>
+    </row>
+    <row r="46">
+      <c r="F46" s="7"/>
+    </row>
+    <row r="47">
+      <c r="F47" s="7"/>
+    </row>
+    <row r="48">
+      <c r="F48" s="7"/>
+    </row>
+    <row r="49">
+      <c r="F49" s="7"/>
+    </row>
+    <row r="50">
+      <c r="F50" s="7"/>
+    </row>
+    <row r="51">
+      <c r="F51" s="7"/>
+    </row>
+    <row r="52">
+      <c r="F52" s="7"/>
+    </row>
+    <row r="53">
+      <c r="F53" s="7"/>
+    </row>
+    <row r="54">
+      <c r="F54" s="7"/>
+    </row>
+    <row r="55">
+      <c r="F55" s="7"/>
+    </row>
+    <row r="56">
+      <c r="F56" s="7"/>
+    </row>
+    <row r="57">
+      <c r="F57" s="7"/>
+    </row>
+    <row r="58">
+      <c r="F58" s="7"/>
+    </row>
+    <row r="59">
+      <c r="F59" s="7"/>
+    </row>
+    <row r="60">
+      <c r="F60" s="7"/>
+    </row>
+    <row r="61">
+      <c r="F61" s="7"/>
+    </row>
+    <row r="62">
+      <c r="F62" s="7"/>
+    </row>
+    <row r="63">
+      <c r="F63" s="7"/>
+    </row>
+    <row r="64">
+      <c r="F64" s="7"/>
+    </row>
+    <row r="65">
+      <c r="F65" s="7"/>
+    </row>
+    <row r="66">
+      <c r="F66" s="7"/>
+    </row>
+    <row r="67">
+      <c r="F67" s="7"/>
+    </row>
+    <row r="68">
+      <c r="F68" s="7"/>
+    </row>
+    <row r="69">
+      <c r="F69" s="7"/>
+    </row>
+    <row r="70">
+      <c r="F70" s="7"/>
+    </row>
+    <row r="71">
+      <c r="F71" s="7"/>
+    </row>
+    <row r="72">
+      <c r="F72" s="7"/>
+    </row>
+    <row r="73">
+      <c r="F73" s="7"/>
+    </row>
+    <row r="74">
+      <c r="F74" s="7"/>
+    </row>
+    <row r="75">
+      <c r="F75" s="7"/>
+    </row>
+    <row r="76">
+      <c r="F76" s="7"/>
+    </row>
+    <row r="77">
+      <c r="F77" s="7"/>
+    </row>
+    <row r="78">
+      <c r="F78" s="7"/>
+    </row>
+    <row r="79">
+      <c r="F79" s="7"/>
+    </row>
+    <row r="80">
+      <c r="F80" s="7"/>
+    </row>
+    <row r="81">
+      <c r="F81" s="7"/>
+    </row>
+    <row r="82">
+      <c r="F82" s="7"/>
+    </row>
+    <row r="83">
+      <c r="F83" s="7"/>
+    </row>
+    <row r="84">
+      <c r="F84" s="7"/>
+    </row>
+    <row r="85">
+      <c r="F85" s="7"/>
+    </row>
+    <row r="86">
+      <c r="F86" s="7"/>
+    </row>
+    <row r="87">
+      <c r="F87" s="7"/>
+    </row>
+    <row r="88">
+      <c r="F88" s="7"/>
+    </row>
+    <row r="89">
+      <c r="F89" s="7"/>
+    </row>
+    <row r="90">
+      <c r="F90" s="7"/>
+    </row>
+    <row r="91">
+      <c r="F91" s="7"/>
+    </row>
+    <row r="92">
+      <c r="F92" s="7"/>
+    </row>
+    <row r="93">
+      <c r="F93" s="7"/>
+    </row>
+    <row r="94">
+      <c r="F94" s="7"/>
+    </row>
+    <row r="95">
+      <c r="F95" s="7"/>
+    </row>
+    <row r="96">
+      <c r="F96" s="7"/>
+    </row>
+    <row r="97">
+      <c r="F97" s="7"/>
+    </row>
+    <row r="98">
+      <c r="F98" s="7"/>
+    </row>
+    <row r="99">
+      <c r="F99" s="7"/>
+    </row>
+    <row r="100">
+      <c r="F100" s="7"/>
+    </row>
+    <row r="101">
+      <c r="F101" s="7"/>
+    </row>
+    <row r="102">
+      <c r="F102" s="7"/>
+    </row>
+    <row r="103">
+      <c r="F103" s="7"/>
+    </row>
+    <row r="104">
+      <c r="F104" s="7"/>
+    </row>
+    <row r="105">
+      <c r="F105" s="7"/>
+    </row>
+    <row r="106">
+      <c r="F106" s="7"/>
+    </row>
+    <row r="107">
+      <c r="F107" s="7"/>
+    </row>
+    <row r="108">
+      <c r="F108" s="7"/>
+    </row>
+    <row r="109">
+      <c r="F109" s="7"/>
+    </row>
+    <row r="110">
+      <c r="F110" s="7"/>
+    </row>
+    <row r="111">
+      <c r="F111" s="7"/>
+    </row>
+    <row r="112">
+      <c r="F112" s="7"/>
+    </row>
+    <row r="113">
+      <c r="F113" s="7"/>
+    </row>
+    <row r="114">
+      <c r="F114" s="7"/>
+    </row>
+    <row r="115">
+      <c r="F115" s="7"/>
+    </row>
+    <row r="116">
+      <c r="F116" s="7"/>
+    </row>
+    <row r="117">
+      <c r="F117" s="7"/>
+    </row>
+    <row r="118">
+      <c r="F118" s="7"/>
+    </row>
+    <row r="119">
+      <c r="F119" s="7"/>
+    </row>
+    <row r="120">
+      <c r="F120" s="7"/>
+    </row>
+    <row r="121">
+      <c r="F121" s="7"/>
+    </row>
+    <row r="122">
+      <c r="F122" s="7"/>
+    </row>
+    <row r="123">
+      <c r="F123" s="7"/>
+    </row>
+    <row r="124">
+      <c r="F124" s="7"/>
+    </row>
+    <row r="125">
+      <c r="F125" s="7"/>
+    </row>
+    <row r="126">
+      <c r="F126" s="7"/>
+    </row>
+    <row r="127">
+      <c r="F127" s="7"/>
+    </row>
+    <row r="128">
+      <c r="F128" s="7"/>
+    </row>
+    <row r="129">
+      <c r="F129" s="7"/>
+    </row>
+    <row r="130">
+      <c r="F130" s="7"/>
+    </row>
+    <row r="131">
+      <c r="F131" s="7"/>
+    </row>
+    <row r="132">
+      <c r="F132" s="7"/>
+    </row>
+    <row r="133">
+      <c r="F133" s="7"/>
+    </row>
+    <row r="134">
+      <c r="F134" s="7"/>
+    </row>
+    <row r="135">
+      <c r="F135" s="7"/>
+    </row>
+    <row r="136">
+      <c r="F136" s="7"/>
+    </row>
+    <row r="137">
+      <c r="F137" s="7"/>
+    </row>
+    <row r="138">
+      <c r="F138" s="7"/>
+    </row>
+    <row r="139">
+      <c r="F139" s="7"/>
+    </row>
+    <row r="140">
+      <c r="F140" s="7"/>
+    </row>
+    <row r="141">
+      <c r="F141" s="7"/>
+    </row>
+    <row r="142">
+      <c r="F142" s="7"/>
+    </row>
+    <row r="143">
+      <c r="F143" s="7"/>
+    </row>
+    <row r="144">
+      <c r="F144" s="7"/>
+    </row>
+    <row r="145">
+      <c r="F145" s="7"/>
+    </row>
+    <row r="146">
+      <c r="F146" s="7"/>
+    </row>
+    <row r="147">
+      <c r="F147" s="7"/>
+    </row>
+    <row r="148">
+      <c r="F148" s="7"/>
+    </row>
+    <row r="149">
+      <c r="F149" s="7"/>
+    </row>
+    <row r="150">
+      <c r="F150" s="7"/>
+    </row>
+    <row r="151">
+      <c r="F151" s="7"/>
+    </row>
+    <row r="152">
+      <c r="F152" s="7"/>
+    </row>
+    <row r="153">
+      <c r="F153" s="7"/>
+    </row>
+    <row r="154">
+      <c r="F154" s="7"/>
+    </row>
+    <row r="155">
+      <c r="F155" s="7"/>
+    </row>
+    <row r="156">
+      <c r="F156" s="7"/>
+    </row>
+    <row r="157">
+      <c r="F157" s="7"/>
+    </row>
+    <row r="158">
+      <c r="F158" s="7"/>
+    </row>
+    <row r="159">
+      <c r="F159" s="7"/>
+    </row>
+    <row r="160">
+      <c r="F160" s="7"/>
+    </row>
+    <row r="161">
+      <c r="F161" s="7"/>
+    </row>
+    <row r="162">
+      <c r="F162" s="7"/>
+    </row>
+    <row r="163">
+      <c r="F163" s="7"/>
+    </row>
+    <row r="164">
+      <c r="F164" s="7"/>
+    </row>
+    <row r="165">
+      <c r="F165" s="7"/>
+    </row>
+    <row r="166">
+      <c r="F166" s="7"/>
+    </row>
+    <row r="167">
+      <c r="F167" s="7"/>
+    </row>
+    <row r="168">
+      <c r="F168" s="7"/>
+    </row>
+    <row r="169">
+      <c r="F169" s="7"/>
+    </row>
+    <row r="170">
+      <c r="F170" s="7"/>
+    </row>
+    <row r="171">
+      <c r="F171" s="7"/>
+    </row>
+    <row r="172">
+      <c r="F172" s="7"/>
+    </row>
+    <row r="173">
+      <c r="F173" s="7"/>
+    </row>
+    <row r="174">
+      <c r="F174" s="7"/>
+    </row>
+    <row r="175">
+      <c r="F175" s="7"/>
+    </row>
+    <row r="176">
+      <c r="F176" s="7"/>
+    </row>
+    <row r="177">
+      <c r="F177" s="7"/>
+    </row>
+    <row r="178">
+      <c r="F178" s="7"/>
+    </row>
+    <row r="179">
+      <c r="F179" s="7"/>
+    </row>
+    <row r="180">
+      <c r="F180" s="7"/>
+    </row>
+    <row r="181">
+      <c r="F181" s="7"/>
+    </row>
+    <row r="182">
+      <c r="F182" s="7"/>
+    </row>
+    <row r="183">
+      <c r="F183" s="7"/>
+    </row>
+    <row r="184">
+      <c r="F184" s="7"/>
+    </row>
+    <row r="185">
+      <c r="F185" s="7"/>
+    </row>
+    <row r="186">
+      <c r="F186" s="7"/>
+    </row>
+    <row r="187">
+      <c r="F187" s="7"/>
+    </row>
+    <row r="188">
+      <c r="F188" s="7"/>
+    </row>
+    <row r="189">
+      <c r="F189" s="7"/>
+    </row>
+    <row r="190">
+      <c r="F190" s="7"/>
+    </row>
+    <row r="191">
+      <c r="F191" s="7"/>
+    </row>
+    <row r="192">
+      <c r="F192" s="7"/>
+    </row>
+    <row r="193">
+      <c r="F193" s="7"/>
+    </row>
+    <row r="194">
+      <c r="F194" s="7"/>
+    </row>
+    <row r="195">
+      <c r="F195" s="7"/>
+    </row>
+    <row r="196">
+      <c r="F196" s="7"/>
+    </row>
+    <row r="197">
+      <c r="F197" s="7"/>
+    </row>
+    <row r="198">
+      <c r="F198" s="7"/>
+    </row>
+    <row r="199">
+      <c r="F199" s="7"/>
+    </row>
+    <row r="200">
+      <c r="F200" s="7"/>
+    </row>
+    <row r="201">
+      <c r="F201" s="7"/>
+    </row>
+    <row r="202">
+      <c r="F202" s="7"/>
+    </row>
+    <row r="203">
+      <c r="F203" s="7"/>
+    </row>
+    <row r="204">
+      <c r="F204" s="7"/>
+    </row>
+    <row r="205">
+      <c r="F205" s="7"/>
+    </row>
+    <row r="206">
+      <c r="F206" s="7"/>
+    </row>
+    <row r="207">
+      <c r="F207" s="7"/>
+    </row>
+    <row r="208">
+      <c r="F208" s="7"/>
+    </row>
+    <row r="209">
+      <c r="F209" s="7"/>
+    </row>
+    <row r="210">
+      <c r="F210" s="7"/>
+    </row>
+    <row r="211">
+      <c r="F211" s="7"/>
+    </row>
+    <row r="212">
+      <c r="F212" s="7"/>
+    </row>
+    <row r="213">
+      <c r="F213" s="7"/>
+    </row>
+    <row r="214">
+      <c r="F214" s="7"/>
+    </row>
+    <row r="215">
+      <c r="F215" s="7"/>
+    </row>
+    <row r="216">
+      <c r="F216" s="7"/>
+    </row>
+    <row r="217">
+      <c r="F217" s="7"/>
+    </row>
+    <row r="218">
+      <c r="F218" s="7"/>
+    </row>
+    <row r="219">
+      <c r="F219" s="7"/>
+    </row>
+    <row r="220">
+      <c r="F220" s="7"/>
+    </row>
+    <row r="221">
+      <c r="F221" s="7"/>
+    </row>
+    <row r="222">
+      <c r="F222" s="7"/>
+    </row>
+    <row r="223">
+      <c r="F223" s="7"/>
+    </row>
+    <row r="224">
+      <c r="F224" s="7"/>
+    </row>
+    <row r="225">
+      <c r="F225" s="7"/>
+    </row>
+    <row r="226">
+      <c r="F226" s="7"/>
+    </row>
+    <row r="227">
+      <c r="F227" s="7"/>
+    </row>
+    <row r="228">
+      <c r="F228" s="7"/>
+    </row>
+    <row r="229">
+      <c r="F229" s="7"/>
+    </row>
+    <row r="230">
+      <c r="F230" s="7"/>
+    </row>
+    <row r="231">
+      <c r="F231" s="7"/>
+    </row>
+    <row r="232">
+      <c r="F232" s="7"/>
+    </row>
+    <row r="233">
+      <c r="F233" s="7"/>
+    </row>
+    <row r="234">
+      <c r="F234" s="7"/>
+    </row>
+    <row r="235">
+      <c r="F235" s="7"/>
+    </row>
+    <row r="236">
+      <c r="F236" s="7"/>
+    </row>
+    <row r="237">
+      <c r="F237" s="7"/>
+    </row>
+    <row r="238">
+      <c r="F238" s="7"/>
+    </row>
+    <row r="239">
+      <c r="F239" s="7"/>
+    </row>
+    <row r="240">
+      <c r="F240" s="7"/>
+    </row>
+    <row r="241">
+      <c r="F241" s="7"/>
+    </row>
+    <row r="242">
+      <c r="F242" s="7"/>
+    </row>
+    <row r="243">
+      <c r="F243" s="7"/>
+    </row>
+    <row r="244">
+      <c r="F244" s="7"/>
+    </row>
+    <row r="245">
+      <c r="F245" s="7"/>
+    </row>
+    <row r="246">
+      <c r="F246" s="7"/>
+    </row>
+    <row r="247">
+      <c r="F247" s="7"/>
+    </row>
+    <row r="248">
+      <c r="F248" s="7"/>
+    </row>
+    <row r="249">
+      <c r="F249" s="7"/>
+    </row>
+    <row r="250">
+      <c r="F250" s="7"/>
+    </row>
+    <row r="251">
+      <c r="F251" s="7"/>
+    </row>
+    <row r="252">
+      <c r="F252" s="7"/>
+    </row>
+    <row r="253">
+      <c r="F253" s="7"/>
+    </row>
+    <row r="254">
+      <c r="F254" s="7"/>
+    </row>
+    <row r="255">
+      <c r="F255" s="7"/>
+    </row>
+    <row r="256">
+      <c r="F256" s="7"/>
+    </row>
+    <row r="257">
+      <c r="F257" s="7"/>
+    </row>
+    <row r="258">
+      <c r="F258" s="7"/>
+    </row>
+    <row r="259">
+      <c r="F259" s="7"/>
+    </row>
+    <row r="260">
+      <c r="F260" s="7"/>
+    </row>
+    <row r="261">
+      <c r="F261" s="7"/>
+    </row>
+    <row r="262">
+      <c r="F262" s="7"/>
+    </row>
+    <row r="263">
+      <c r="F263" s="7"/>
+    </row>
+    <row r="264">
+      <c r="F264" s="7"/>
+    </row>
+    <row r="265">
+      <c r="F265" s="7"/>
+    </row>
+    <row r="266">
+      <c r="F266" s="7"/>
+    </row>
+    <row r="267">
+      <c r="F267" s="7"/>
+    </row>
+    <row r="268">
+      <c r="F268" s="7"/>
+    </row>
+    <row r="269">
+      <c r="F269" s="7"/>
+    </row>
+    <row r="270">
+      <c r="F270" s="7"/>
+    </row>
+    <row r="271">
+      <c r="F271" s="7"/>
+    </row>
+    <row r="272">
+      <c r="F272" s="7"/>
+    </row>
+    <row r="273">
+      <c r="F273" s="7"/>
+    </row>
+    <row r="274">
+      <c r="F274" s="7"/>
+    </row>
+    <row r="275">
+      <c r="F275" s="7"/>
+    </row>
+    <row r="276">
+      <c r="F276" s="7"/>
+    </row>
+    <row r="277">
+      <c r="F277" s="7"/>
+    </row>
+    <row r="278">
+      <c r="F278" s="7"/>
+    </row>
+    <row r="279">
+      <c r="F279" s="7"/>
+    </row>
+    <row r="280">
+      <c r="F280" s="7"/>
+    </row>
+    <row r="281">
+      <c r="F281" s="7"/>
+    </row>
+    <row r="282">
+      <c r="F282" s="7"/>
+    </row>
+    <row r="283">
+      <c r="F283" s="7"/>
+    </row>
+    <row r="284">
+      <c r="F284" s="7"/>
+    </row>
+    <row r="285">
+      <c r="F285" s="7"/>
+    </row>
+    <row r="286">
+      <c r="F286" s="7"/>
+    </row>
+    <row r="287">
+      <c r="F287" s="7"/>
+    </row>
+    <row r="288">
+      <c r="F288" s="7"/>
+    </row>
+    <row r="289">
+      <c r="F289" s="7"/>
+    </row>
+    <row r="290">
+      <c r="F290" s="7"/>
+    </row>
+    <row r="291">
+      <c r="F291" s="7"/>
+    </row>
+    <row r="292">
+      <c r="F292" s="7"/>
+    </row>
+    <row r="293">
+      <c r="F293" s="7"/>
+    </row>
+    <row r="294">
+      <c r="F294" s="7"/>
+    </row>
+    <row r="295">
+      <c r="F295" s="7"/>
+    </row>
+    <row r="296">
+      <c r="F296" s="7"/>
+    </row>
+    <row r="297">
+      <c r="F297" s="7"/>
+    </row>
+    <row r="298">
+      <c r="F298" s="7"/>
+    </row>
+    <row r="299">
+      <c r="F299" s="7"/>
+    </row>
+    <row r="300">
+      <c r="F300" s="7"/>
+    </row>
+    <row r="301">
+      <c r="F301" s="7"/>
+    </row>
+    <row r="302">
+      <c r="F302" s="7"/>
+    </row>
+    <row r="303">
+      <c r="F303" s="7"/>
+    </row>
+    <row r="304">
+      <c r="F304" s="7"/>
+    </row>
+    <row r="305">
+      <c r="F305" s="7"/>
+    </row>
+    <row r="306">
+      <c r="F306" s="7"/>
+    </row>
+    <row r="307">
+      <c r="F307" s="7"/>
+    </row>
+    <row r="308">
+      <c r="F308" s="7"/>
+    </row>
+    <row r="309">
+      <c r="F309" s="7"/>
+    </row>
+    <row r="310">
+      <c r="F310" s="7"/>
+    </row>
+    <row r="311">
+      <c r="F311" s="7"/>
+    </row>
+    <row r="312">
+      <c r="F312" s="7"/>
+    </row>
+    <row r="313">
+      <c r="F313" s="7"/>
+    </row>
+    <row r="314">
+      <c r="F314" s="7"/>
+    </row>
+    <row r="315">
+      <c r="F315" s="7"/>
+    </row>
+    <row r="316">
+      <c r="F316" s="7"/>
+    </row>
+    <row r="317">
+      <c r="F317" s="7"/>
+    </row>
+    <row r="318">
+      <c r="F318" s="7"/>
+    </row>
+    <row r="319">
+      <c r="F319" s="7"/>
+    </row>
+    <row r="320">
+      <c r="F320" s="7"/>
+    </row>
+    <row r="321">
+      <c r="F321" s="7"/>
+    </row>
+    <row r="322">
+      <c r="F322" s="7"/>
+    </row>
+    <row r="323">
+      <c r="F323" s="7"/>
+    </row>
+    <row r="324">
+      <c r="F324" s="7"/>
+    </row>
+    <row r="325">
+      <c r="F325" s="7"/>
+    </row>
+    <row r="326">
+      <c r="F326" s="7"/>
+    </row>
+    <row r="327">
+      <c r="F327" s="7"/>
+    </row>
+    <row r="328">
+      <c r="F328" s="7"/>
+    </row>
+    <row r="329">
+      <c r="F329" s="7"/>
+    </row>
+    <row r="330">
+      <c r="F330" s="7"/>
+    </row>
+    <row r="331">
+      <c r="F331" s="7"/>
+    </row>
+    <row r="332">
+      <c r="F332" s="7"/>
+    </row>
+    <row r="333">
+      <c r="F333" s="7"/>
+    </row>
+    <row r="334">
+      <c r="F334" s="7"/>
+    </row>
+    <row r="335">
+      <c r="F335" s="7"/>
+    </row>
+    <row r="336">
+      <c r="F336" s="7"/>
+    </row>
+    <row r="337">
+      <c r="F337" s="7"/>
+    </row>
+    <row r="338">
+      <c r="F338" s="7"/>
+    </row>
+    <row r="339">
+      <c r="F339" s="7"/>
+    </row>
+    <row r="340">
+      <c r="F340" s="7"/>
+    </row>
+    <row r="341">
+      <c r="F341" s="7"/>
+    </row>
+    <row r="342">
+      <c r="F342" s="7"/>
+    </row>
+    <row r="343">
+      <c r="F343" s="7"/>
+    </row>
+    <row r="344">
+      <c r="F344" s="7"/>
+    </row>
+    <row r="345">
+      <c r="F345" s="7"/>
+    </row>
+    <row r="346">
+      <c r="F346" s="7"/>
+    </row>
+    <row r="347">
+      <c r="F347" s="7"/>
+    </row>
+    <row r="348">
+      <c r="F348" s="7"/>
+    </row>
+    <row r="349">
+      <c r="F349" s="7"/>
+    </row>
+    <row r="350">
+      <c r="F350" s="7"/>
+    </row>
+    <row r="351">
+      <c r="F351" s="7"/>
+    </row>
+    <row r="352">
+      <c r="F352" s="7"/>
+    </row>
+    <row r="353">
+      <c r="F353" s="7"/>
+    </row>
+    <row r="354">
+      <c r="F354" s="7"/>
+    </row>
+    <row r="355">
+      <c r="F355" s="7"/>
+    </row>
+    <row r="356">
+      <c r="F356" s="7"/>
+    </row>
+    <row r="357">
+      <c r="F357" s="7"/>
+    </row>
+    <row r="358">
+      <c r="F358" s="7"/>
+    </row>
+    <row r="359">
+      <c r="F359" s="7"/>
+    </row>
+    <row r="360">
+      <c r="F360" s="7"/>
+    </row>
+    <row r="361">
+      <c r="F361" s="7"/>
+    </row>
+    <row r="362">
+      <c r="F362" s="7"/>
+    </row>
+    <row r="363">
+      <c r="F363" s="7"/>
+    </row>
+    <row r="364">
+      <c r="F364" s="7"/>
+    </row>
+    <row r="365">
+      <c r="F365" s="7"/>
+    </row>
+    <row r="366">
+      <c r="F366" s="7"/>
+    </row>
+    <row r="367">
+      <c r="F367" s="7"/>
+    </row>
+    <row r="368">
+      <c r="F368" s="7"/>
+    </row>
+    <row r="369">
+      <c r="F369" s="7"/>
+    </row>
+    <row r="370">
+      <c r="F370" s="7"/>
+    </row>
+    <row r="371">
+      <c r="F371" s="7"/>
+    </row>
+    <row r="372">
+      <c r="F372" s="7"/>
+    </row>
+    <row r="373">
+      <c r="F373" s="7"/>
+    </row>
+    <row r="374">
+      <c r="F374" s="7"/>
+    </row>
+    <row r="375">
+      <c r="F375" s="7"/>
+    </row>
+    <row r="376">
+      <c r="F376" s="7"/>
+    </row>
+    <row r="377">
+      <c r="F377" s="7"/>
+    </row>
+    <row r="378">
+      <c r="F378" s="7"/>
+    </row>
+    <row r="379">
+      <c r="F379" s="7"/>
+    </row>
+    <row r="380">
+      <c r="F380" s="7"/>
+    </row>
+    <row r="381">
+      <c r="F381" s="7"/>
+    </row>
+    <row r="382">
+      <c r="F382" s="7"/>
+    </row>
+    <row r="383">
+      <c r="F383" s="7"/>
+    </row>
+    <row r="384">
+      <c r="F384" s="7"/>
+    </row>
+    <row r="385">
+      <c r="F385" s="7"/>
+    </row>
+    <row r="386">
+      <c r="F386" s="7"/>
+    </row>
+    <row r="387">
+      <c r="F387" s="7"/>
+    </row>
+    <row r="388">
+      <c r="F388" s="7"/>
+    </row>
+    <row r="389">
+      <c r="F389" s="7"/>
+    </row>
+    <row r="390">
+      <c r="F390" s="7"/>
+    </row>
+    <row r="391">
+      <c r="F391" s="7"/>
+    </row>
+    <row r="392">
+      <c r="F392" s="7"/>
+    </row>
+    <row r="393">
+      <c r="F393" s="7"/>
+    </row>
+    <row r="394">
+      <c r="F394" s="7"/>
+    </row>
+    <row r="395">
+      <c r="F395" s="7"/>
+    </row>
+    <row r="396">
+      <c r="F396" s="7"/>
+    </row>
+    <row r="397">
+      <c r="F397" s="7"/>
+    </row>
+    <row r="398">
+      <c r="F398" s="7"/>
+    </row>
+    <row r="399">
+      <c r="F399" s="7"/>
+    </row>
+    <row r="400">
+      <c r="F400" s="7"/>
+    </row>
+    <row r="401">
+      <c r="F401" s="7"/>
+    </row>
+    <row r="402">
+      <c r="F402" s="7"/>
+    </row>
+    <row r="403">
+      <c r="F403" s="7"/>
+    </row>
+    <row r="404">
+      <c r="F404" s="7"/>
+    </row>
+    <row r="405">
+      <c r="F405" s="7"/>
+    </row>
+    <row r="406">
+      <c r="F406" s="7"/>
+    </row>
+    <row r="407">
+      <c r="F407" s="7"/>
+    </row>
+    <row r="408">
+      <c r="F408" s="7"/>
+    </row>
+    <row r="409">
+      <c r="F409" s="7"/>
+    </row>
+    <row r="410">
+      <c r="F410" s="7"/>
+    </row>
+    <row r="411">
+      <c r="F411" s="7"/>
+    </row>
+    <row r="412">
+      <c r="F412" s="7"/>
+    </row>
+    <row r="413">
+      <c r="F413" s="7"/>
+    </row>
+    <row r="414">
+      <c r="F414" s="7"/>
+    </row>
+    <row r="415">
+      <c r="F415" s="7"/>
+    </row>
+    <row r="416">
+      <c r="F416" s="7"/>
+    </row>
+    <row r="417">
+      <c r="F417" s="7"/>
+    </row>
+    <row r="418">
+      <c r="F418" s="7"/>
+    </row>
+    <row r="419">
+      <c r="F419" s="7"/>
+    </row>
+    <row r="420">
+      <c r="F420" s="7"/>
+    </row>
+    <row r="421">
+      <c r="F421" s="7"/>
+    </row>
+    <row r="422">
+      <c r="F422" s="7"/>
+    </row>
+    <row r="423">
+      <c r="F423" s="7"/>
+    </row>
+    <row r="424">
+      <c r="F424" s="7"/>
+    </row>
+    <row r="425">
+      <c r="F425" s="7"/>
+    </row>
+    <row r="426">
+      <c r="F426" s="7"/>
+    </row>
+    <row r="427">
+      <c r="F427" s="7"/>
+    </row>
+    <row r="428">
+      <c r="F428" s="7"/>
+    </row>
+    <row r="429">
+      <c r="F429" s="7"/>
+    </row>
+    <row r="430">
+      <c r="F430" s="7"/>
+    </row>
+    <row r="431">
+      <c r="F431" s="7"/>
+    </row>
+    <row r="432">
+      <c r="F432" s="7"/>
+    </row>
+    <row r="433">
+      <c r="F433" s="7"/>
+    </row>
+    <row r="434">
+      <c r="F434" s="7"/>
+    </row>
+    <row r="435">
+      <c r="F435" s="7"/>
+    </row>
+    <row r="436">
+      <c r="F436" s="7"/>
+    </row>
+    <row r="437">
+      <c r="F437" s="7"/>
+    </row>
+    <row r="438">
+      <c r="F438" s="7"/>
+    </row>
+    <row r="439">
+      <c r="F439" s="7"/>
+    </row>
+    <row r="440">
+      <c r="F440" s="7"/>
+    </row>
+    <row r="441">
+      <c r="F441" s="7"/>
+    </row>
+    <row r="442">
+      <c r="F442" s="7"/>
+    </row>
+    <row r="443">
+      <c r="F443" s="7"/>
+    </row>
+    <row r="444">
+      <c r="F444" s="7"/>
+    </row>
+    <row r="445">
+      <c r="F445" s="7"/>
+    </row>
+    <row r="446">
+      <c r="F446" s="7"/>
+    </row>
+    <row r="447">
+      <c r="F447" s="7"/>
+    </row>
+    <row r="448">
+      <c r="F448" s="7"/>
+    </row>
+    <row r="449">
+      <c r="F449" s="7"/>
+    </row>
+    <row r="450">
+      <c r="F450" s="7"/>
+    </row>
+    <row r="451">
+      <c r="F451" s="7"/>
+    </row>
+    <row r="452">
+      <c r="F452" s="7"/>
+    </row>
+    <row r="453">
+      <c r="F453" s="7"/>
+    </row>
+    <row r="454">
+      <c r="F454" s="7"/>
+    </row>
+    <row r="455">
+      <c r="F455" s="7"/>
+    </row>
+    <row r="456">
+      <c r="F456" s="7"/>
+    </row>
+    <row r="457">
+      <c r="F457" s="7"/>
+    </row>
+    <row r="458">
+      <c r="F458" s="7"/>
+    </row>
+    <row r="459">
+      <c r="F459" s="7"/>
+    </row>
+    <row r="460">
+      <c r="F460" s="7"/>
+    </row>
+    <row r="461">
+      <c r="F461" s="7"/>
+    </row>
+    <row r="462">
+      <c r="F462" s="7"/>
+    </row>
+    <row r="463">
+      <c r="F463" s="7"/>
+    </row>
+    <row r="464">
+      <c r="F464" s="7"/>
+    </row>
+    <row r="465">
+      <c r="F465" s="7"/>
+    </row>
+    <row r="466">
+      <c r="F466" s="7"/>
+    </row>
+    <row r="467">
+      <c r="F467" s="7"/>
+    </row>
+    <row r="468">
+      <c r="F468" s="7"/>
+    </row>
+    <row r="469">
+      <c r="F469" s="7"/>
+    </row>
+    <row r="470">
+      <c r="F470" s="7"/>
+    </row>
+    <row r="471">
+      <c r="F471" s="7"/>
+    </row>
+    <row r="472">
+      <c r="F472" s="7"/>
+    </row>
+    <row r="473">
+      <c r="F473" s="7"/>
+    </row>
+    <row r="474">
+      <c r="F474" s="7"/>
+    </row>
+    <row r="475">
+      <c r="F475" s="7"/>
+    </row>
+    <row r="476">
+      <c r="F476" s="7"/>
+    </row>
+    <row r="477">
+      <c r="F477" s="7"/>
+    </row>
+    <row r="478">
+      <c r="F478" s="7"/>
+    </row>
+    <row r="479">
+      <c r="F479" s="7"/>
+    </row>
+    <row r="480">
+      <c r="F480" s="7"/>
+    </row>
+    <row r="481">
+      <c r="F481" s="7"/>
+    </row>
+    <row r="482">
+      <c r="F482" s="7"/>
+    </row>
+    <row r="483">
+      <c r="F483" s="7"/>
+    </row>
+    <row r="484">
+      <c r="F484" s="7"/>
+    </row>
+    <row r="485">
+      <c r="F485" s="7"/>
+    </row>
+    <row r="486">
+      <c r="F486" s="7"/>
+    </row>
+    <row r="487">
+      <c r="F487" s="7"/>
+    </row>
+    <row r="488">
+      <c r="F488" s="7"/>
+    </row>
+    <row r="489">
+      <c r="F489" s="7"/>
+    </row>
+    <row r="490">
+      <c r="F490" s="7"/>
+    </row>
+    <row r="491">
+      <c r="F491" s="7"/>
+    </row>
+    <row r="492">
+      <c r="F492" s="7"/>
+    </row>
+    <row r="493">
+      <c r="F493" s="7"/>
+    </row>
+    <row r="494">
+      <c r="F494" s="7"/>
+    </row>
+    <row r="495">
+      <c r="F495" s="7"/>
+    </row>
+    <row r="496">
+      <c r="F496" s="7"/>
+    </row>
+    <row r="497">
+      <c r="F497" s="7"/>
+    </row>
+    <row r="498">
+      <c r="F498" s="7"/>
+    </row>
+    <row r="499">
+      <c r="F499" s="7"/>
+    </row>
+    <row r="500">
+      <c r="F500" s="7"/>
+    </row>
+    <row r="501">
+      <c r="F501" s="7"/>
+    </row>
+    <row r="502">
+      <c r="F502" s="7"/>
+    </row>
+    <row r="503">
+      <c r="F503" s="7"/>
+    </row>
+    <row r="504">
+      <c r="F504" s="7"/>
+    </row>
+    <row r="505">
+      <c r="F505" s="7"/>
+    </row>
+    <row r="506">
+      <c r="F506" s="7"/>
+    </row>
+    <row r="507">
+      <c r="F507" s="7"/>
+    </row>
+    <row r="508">
+      <c r="F508" s="7"/>
+    </row>
+    <row r="509">
+      <c r="F509" s="7"/>
+    </row>
+    <row r="510">
+      <c r="F510" s="7"/>
+    </row>
+    <row r="511">
+      <c r="F511" s="7"/>
+    </row>
+    <row r="512">
+      <c r="F512" s="7"/>
+    </row>
+    <row r="513">
+      <c r="F513" s="7"/>
+    </row>
+    <row r="514">
+      <c r="F514" s="7"/>
+    </row>
+    <row r="515">
+      <c r="F515" s="7"/>
+    </row>
+    <row r="516">
+      <c r="F516" s="7"/>
+    </row>
+    <row r="517">
+      <c r="F517" s="7"/>
+    </row>
+    <row r="518">
+      <c r="F518" s="7"/>
+    </row>
+    <row r="519">
+      <c r="F519" s="7"/>
+    </row>
+    <row r="520">
+      <c r="F520" s="7"/>
+    </row>
+    <row r="521">
+      <c r="F521" s="7"/>
+    </row>
+    <row r="522">
+      <c r="F522" s="7"/>
+    </row>
+    <row r="523">
+      <c r="F523" s="7"/>
+    </row>
+    <row r="524">
+      <c r="F524" s="7"/>
+    </row>
+    <row r="525">
+      <c r="F525" s="7"/>
+    </row>
+    <row r="526">
+      <c r="F526" s="7"/>
+    </row>
+    <row r="527">
+      <c r="F527" s="7"/>
+    </row>
+    <row r="528">
+      <c r="F528" s="7"/>
+    </row>
+    <row r="529">
+      <c r="F529" s="7"/>
+    </row>
+    <row r="530">
+      <c r="F530" s="7"/>
+    </row>
+    <row r="531">
+      <c r="F531" s="7"/>
+    </row>
+    <row r="532">
+      <c r="F532" s="7"/>
+    </row>
+    <row r="533">
+      <c r="F533" s="7"/>
+    </row>
+    <row r="534">
+      <c r="F534" s="7"/>
+    </row>
+    <row r="535">
+      <c r="F535" s="7"/>
+    </row>
+    <row r="536">
+      <c r="F536" s="7"/>
+    </row>
+    <row r="537">
+      <c r="F537" s="7"/>
+    </row>
+    <row r="538">
+      <c r="F538" s="7"/>
+    </row>
+    <row r="539">
+      <c r="F539" s="7"/>
+    </row>
+    <row r="540">
+      <c r="F540" s="7"/>
+    </row>
+    <row r="541">
+      <c r="F541" s="7"/>
+    </row>
+    <row r="542">
+      <c r="F542" s="7"/>
+    </row>
+    <row r="543">
+      <c r="F543" s="7"/>
+    </row>
+    <row r="544">
+      <c r="F544" s="7"/>
+    </row>
+    <row r="545">
+      <c r="F545" s="7"/>
+    </row>
+    <row r="546">
+      <c r="F546" s="7"/>
+    </row>
+    <row r="547">
+      <c r="F547" s="7"/>
+    </row>
+    <row r="548">
+      <c r="F548" s="7"/>
+    </row>
+    <row r="549">
+      <c r="F549" s="7"/>
+    </row>
+    <row r="550">
+      <c r="F550" s="7"/>
+    </row>
+    <row r="551">
+      <c r="F551" s="7"/>
+    </row>
+    <row r="552">
+      <c r="F552" s="7"/>
+    </row>
+    <row r="553">
+      <c r="F553" s="7"/>
+    </row>
+    <row r="554">
+      <c r="F554" s="7"/>
+    </row>
+    <row r="555">
+      <c r="F555" s="7"/>
+    </row>
+    <row r="556">
+      <c r="F556" s="7"/>
+    </row>
+    <row r="557">
+      <c r="F557" s="7"/>
+    </row>
+    <row r="558">
+      <c r="F558" s="7"/>
+    </row>
+    <row r="559">
+      <c r="F559" s="7"/>
+    </row>
+    <row r="560">
+      <c r="F560" s="7"/>
+    </row>
+    <row r="561">
+      <c r="F561" s="7"/>
+    </row>
+    <row r="562">
+      <c r="F562" s="7"/>
+    </row>
+    <row r="563">
+      <c r="F563" s="7"/>
+    </row>
+    <row r="564">
+      <c r="F564" s="7"/>
+    </row>
+    <row r="565">
+      <c r="F565" s="7"/>
+    </row>
+    <row r="566">
+      <c r="F566" s="7"/>
+    </row>
+    <row r="567">
+      <c r="F567" s="7"/>
+    </row>
+    <row r="568">
+      <c r="F568" s="7"/>
+    </row>
+    <row r="569">
+      <c r="F569" s="7"/>
+    </row>
+    <row r="570">
+      <c r="F570" s="7"/>
+    </row>
+    <row r="571">
+      <c r="F571" s="7"/>
+    </row>
+    <row r="572">
+      <c r="F572" s="7"/>
+    </row>
+    <row r="573">
+      <c r="F573" s="7"/>
+    </row>
+    <row r="574">
+      <c r="F574" s="7"/>
+    </row>
+    <row r="575">
+      <c r="F575" s="7"/>
+    </row>
+    <row r="576">
+      <c r="F576" s="7"/>
+    </row>
+    <row r="577">
+      <c r="F577" s="7"/>
+    </row>
+    <row r="578">
+      <c r="F578" s="7"/>
+    </row>
+    <row r="579">
+      <c r="F579" s="7"/>
+    </row>
+    <row r="580">
+      <c r="F580" s="7"/>
+    </row>
+    <row r="581">
+      <c r="F581" s="7"/>
+    </row>
+    <row r="582">
+      <c r="F582" s="7"/>
+    </row>
+    <row r="583">
+      <c r="F583" s="7"/>
+    </row>
+    <row r="584">
+      <c r="F584" s="7"/>
+    </row>
+    <row r="585">
+      <c r="F585" s="7"/>
+    </row>
+    <row r="586">
+      <c r="F586" s="7"/>
+    </row>
+    <row r="587">
+      <c r="F587" s="7"/>
+    </row>
+    <row r="588">
+      <c r="F588" s="7"/>
+    </row>
+    <row r="589">
+      <c r="F589" s="7"/>
+    </row>
+    <row r="590">
+      <c r="F590" s="7"/>
+    </row>
+    <row r="591">
+      <c r="F591" s="7"/>
+    </row>
+    <row r="592">
+      <c r="F592" s="7"/>
+    </row>
+    <row r="593">
+      <c r="F593" s="7"/>
+    </row>
+    <row r="594">
+      <c r="F594" s="7"/>
+    </row>
+    <row r="595">
+      <c r="F595" s="7"/>
+    </row>
+    <row r="596">
+      <c r="F596" s="7"/>
+    </row>
+    <row r="597">
+      <c r="F597" s="7"/>
+    </row>
+    <row r="598">
+      <c r="F598" s="7"/>
+    </row>
+    <row r="599">
+      <c r="F599" s="7"/>
+    </row>
+    <row r="600">
+      <c r="F600" s="7"/>
+    </row>
+    <row r="601">
+      <c r="F601" s="7"/>
+    </row>
+    <row r="602">
+      <c r="F602" s="7"/>
+    </row>
+    <row r="603">
+      <c r="F603" s="7"/>
+    </row>
+    <row r="604">
+      <c r="F604" s="7"/>
+    </row>
+    <row r="605">
+      <c r="F605" s="7"/>
+    </row>
+    <row r="606">
+      <c r="F606" s="7"/>
+    </row>
+    <row r="607">
+      <c r="F607" s="7"/>
+    </row>
+    <row r="608">
+      <c r="F608" s="7"/>
+    </row>
+    <row r="609">
+      <c r="F609" s="7"/>
+    </row>
+    <row r="610">
+      <c r="F610" s="7"/>
+    </row>
+    <row r="611">
+      <c r="F611" s="7"/>
+    </row>
+    <row r="612">
+      <c r="F612" s="7"/>
+    </row>
+    <row r="613">
+      <c r="F613" s="7"/>
+    </row>
+    <row r="614">
+      <c r="F614" s="7"/>
+    </row>
+    <row r="615">
+      <c r="F615" s="7"/>
+    </row>
+    <row r="616">
+      <c r="F616" s="7"/>
+    </row>
+    <row r="617">
+      <c r="F617" s="7"/>
+    </row>
+    <row r="618">
+      <c r="F618" s="7"/>
+    </row>
+    <row r="619">
+      <c r="F619" s="7"/>
+    </row>
+    <row r="620">
+      <c r="F620" s="7"/>
+    </row>
+    <row r="621">
+      <c r="F621" s="7"/>
+    </row>
+    <row r="622">
+      <c r="F622" s="7"/>
+    </row>
+    <row r="623">
+      <c r="F623" s="7"/>
+    </row>
+    <row r="624">
+      <c r="F624" s="7"/>
+    </row>
+    <row r="625">
+      <c r="F625" s="7"/>
+    </row>
+    <row r="626">
+      <c r="F626" s="7"/>
+    </row>
+    <row r="627">
+      <c r="F627" s="7"/>
+    </row>
+    <row r="628">
+      <c r="F628" s="7"/>
+    </row>
+    <row r="629">
+      <c r="F629" s="7"/>
+    </row>
+    <row r="630">
+      <c r="F630" s="7"/>
+    </row>
+    <row r="631">
+      <c r="F631" s="7"/>
+    </row>
+    <row r="632">
+      <c r="F632" s="7"/>
+    </row>
+    <row r="633">
+      <c r="F633" s="7"/>
+    </row>
+    <row r="634">
+      <c r="F634" s="7"/>
+    </row>
+    <row r="635">
+      <c r="F635" s="7"/>
+    </row>
+    <row r="636">
+      <c r="F636" s="7"/>
+    </row>
+    <row r="637">
+      <c r="F637" s="7"/>
+    </row>
+    <row r="638">
+      <c r="F638" s="7"/>
+    </row>
+    <row r="639">
+      <c r="F639" s="7"/>
+    </row>
+    <row r="640">
+      <c r="F640" s="7"/>
+    </row>
+    <row r="641">
+      <c r="F641" s="7"/>
+    </row>
+    <row r="642">
+      <c r="F642" s="7"/>
+    </row>
+    <row r="643">
+      <c r="F643" s="7"/>
+    </row>
+    <row r="644">
+      <c r="F644" s="7"/>
+    </row>
+    <row r="645">
+      <c r="F645" s="7"/>
+    </row>
+    <row r="646">
+      <c r="F646" s="7"/>
+    </row>
+    <row r="647">
+      <c r="F647" s="7"/>
+    </row>
+    <row r="648">
+      <c r="F648" s="7"/>
+    </row>
+    <row r="649">
+      <c r="F649" s="7"/>
+    </row>
+    <row r="650">
+      <c r="F650" s="7"/>
+    </row>
+    <row r="651">
+      <c r="F651" s="7"/>
+    </row>
+    <row r="652">
+      <c r="F652" s="7"/>
+    </row>
+    <row r="653">
+      <c r="F653" s="7"/>
+    </row>
+    <row r="654">
+      <c r="F654" s="7"/>
+    </row>
+    <row r="655">
+      <c r="F655" s="7"/>
+    </row>
+    <row r="656">
+      <c r="F656" s="7"/>
+    </row>
+    <row r="657">
+      <c r="F657" s="7"/>
+    </row>
+    <row r="658">
+      <c r="F658" s="7"/>
+    </row>
+    <row r="659">
+      <c r="F659" s="7"/>
+    </row>
+    <row r="660">
+      <c r="F660" s="7"/>
+    </row>
+    <row r="661">
+      <c r="F661" s="7"/>
+    </row>
+    <row r="662">
+      <c r="F662" s="7"/>
+    </row>
+    <row r="663">
+      <c r="F663" s="7"/>
+    </row>
+    <row r="664">
+      <c r="F664" s="7"/>
+    </row>
+    <row r="665">
+      <c r="F665" s="7"/>
+    </row>
+    <row r="666">
+      <c r="F666" s="7"/>
+    </row>
+    <row r="667">
+      <c r="F667" s="7"/>
+    </row>
+    <row r="668">
+      <c r="F668" s="7"/>
+    </row>
+    <row r="669">
+      <c r="F669" s="7"/>
+    </row>
+    <row r="670">
+      <c r="F670" s="7"/>
+    </row>
+    <row r="671">
+      <c r="F671" s="7"/>
+    </row>
+    <row r="672">
+      <c r="F672" s="7"/>
+    </row>
+    <row r="673">
+      <c r="F673" s="7"/>
+    </row>
+    <row r="674">
+      <c r="F674" s="7"/>
+    </row>
+    <row r="675">
+      <c r="F675" s="7"/>
+    </row>
+    <row r="676">
+      <c r="F676" s="7"/>
+    </row>
+    <row r="677">
+      <c r="F677" s="7"/>
+    </row>
+    <row r="678">
+      <c r="F678" s="7"/>
+    </row>
+    <row r="679">
+      <c r="F679" s="7"/>
+    </row>
+    <row r="680">
+      <c r="F680" s="7"/>
+    </row>
+    <row r="681">
+      <c r="F681" s="7"/>
+    </row>
+    <row r="682">
+      <c r="F682" s="7"/>
+    </row>
+    <row r="683">
+      <c r="F683" s="7"/>
+    </row>
+    <row r="684">
+      <c r="F684" s="7"/>
+    </row>
+    <row r="685">
+      <c r="F685" s="7"/>
+    </row>
+    <row r="686">
+      <c r="F686" s="7"/>
+    </row>
+    <row r="687">
+      <c r="F687" s="7"/>
+    </row>
+    <row r="688">
+      <c r="F688" s="7"/>
+    </row>
+    <row r="689">
+      <c r="F689" s="7"/>
+    </row>
+    <row r="690">
+      <c r="F690" s="7"/>
+    </row>
+    <row r="691">
+      <c r="F691" s="7"/>
+    </row>
+    <row r="692">
+      <c r="F692" s="7"/>
+    </row>
+    <row r="693">
+      <c r="F693" s="7"/>
+    </row>
+    <row r="694">
+      <c r="F694" s="7"/>
+    </row>
+    <row r="695">
+      <c r="F695" s="7"/>
+    </row>
+    <row r="696">
+      <c r="F696" s="7"/>
+    </row>
+    <row r="697">
+      <c r="F697" s="7"/>
+    </row>
+    <row r="698">
+      <c r="F698" s="7"/>
+    </row>
+    <row r="699">
+      <c r="F699" s="7"/>
+    </row>
+    <row r="700">
+      <c r="F700" s="7"/>
+    </row>
+    <row r="701">
+      <c r="F701" s="7"/>
+    </row>
+    <row r="702">
+      <c r="F702" s="7"/>
+    </row>
+    <row r="703">
+      <c r="F703" s="7"/>
+    </row>
+    <row r="704">
+      <c r="F704" s="7"/>
+    </row>
+    <row r="705">
+      <c r="F705" s="7"/>
+    </row>
+    <row r="706">
+      <c r="F706" s="7"/>
+    </row>
+    <row r="707">
+      <c r="F707" s="7"/>
+    </row>
+    <row r="708">
+      <c r="F708" s="7"/>
+    </row>
+    <row r="709">
+      <c r="F709" s="7"/>
+    </row>
+    <row r="710">
+      <c r="F710" s="7"/>
+    </row>
+    <row r="711">
+      <c r="F711" s="7"/>
+    </row>
+    <row r="712">
+      <c r="F712" s="7"/>
+    </row>
+    <row r="713">
+      <c r="F713" s="7"/>
+    </row>
+    <row r="714">
+      <c r="F714" s="7"/>
+    </row>
+    <row r="715">
+      <c r="F715" s="7"/>
+    </row>
+    <row r="716">
+      <c r="F716" s="7"/>
+    </row>
+    <row r="717">
+      <c r="F717" s="7"/>
+    </row>
+    <row r="718">
+      <c r="F718" s="7"/>
+    </row>
+    <row r="719">
+      <c r="F719" s="7"/>
+    </row>
+    <row r="720">
+      <c r="F720" s="7"/>
+    </row>
+    <row r="721">
+      <c r="F721" s="7"/>
+    </row>
+    <row r="722">
+      <c r="F722" s="7"/>
+    </row>
+    <row r="723">
+      <c r="F723" s="7"/>
+    </row>
+    <row r="724">
+      <c r="F724" s="7"/>
+    </row>
+    <row r="725">
+      <c r="F725" s="7"/>
+    </row>
+    <row r="726">
+      <c r="F726" s="7"/>
+    </row>
+    <row r="727">
+      <c r="F727" s="7"/>
+    </row>
+    <row r="728">
+      <c r="F728" s="7"/>
+    </row>
+    <row r="729">
+      <c r="F729" s="7"/>
+    </row>
+    <row r="730">
+      <c r="F730" s="7"/>
+    </row>
+    <row r="731">
+      <c r="F731" s="7"/>
+    </row>
+    <row r="732">
+      <c r="F732" s="7"/>
+    </row>
+    <row r="733">
+      <c r="F733" s="7"/>
+    </row>
+    <row r="734">
+      <c r="F734" s="7"/>
+    </row>
+    <row r="735">
+      <c r="F735" s="7"/>
+    </row>
+    <row r="736">
+      <c r="F736" s="7"/>
+    </row>
+    <row r="737">
+      <c r="F737" s="7"/>
+    </row>
+    <row r="738">
+      <c r="F738" s="7"/>
+    </row>
+    <row r="739">
+      <c r="F739" s="7"/>
+    </row>
+    <row r="740">
+      <c r="F740" s="7"/>
+    </row>
+    <row r="741">
+      <c r="F741" s="7"/>
+    </row>
+    <row r="742">
+      <c r="F742" s="7"/>
+    </row>
+    <row r="743">
+      <c r="F743" s="7"/>
+    </row>
+    <row r="744">
+      <c r="F744" s="7"/>
+    </row>
+    <row r="745">
+      <c r="F745" s="7"/>
+    </row>
+    <row r="746">
+      <c r="F746" s="7"/>
+    </row>
+    <row r="747">
+      <c r="F747" s="7"/>
+    </row>
+    <row r="748">
+      <c r="F748" s="7"/>
+    </row>
+    <row r="749">
+      <c r="F749" s="7"/>
+    </row>
+    <row r="750">
+      <c r="F750" s="7"/>
+    </row>
+    <row r="751">
+      <c r="F751" s="7"/>
+    </row>
+    <row r="752">
+      <c r="F752" s="7"/>
+    </row>
+    <row r="753">
+      <c r="F753" s="7"/>
+    </row>
+    <row r="754">
+      <c r="F754" s="7"/>
+    </row>
+    <row r="755">
+      <c r="F755" s="7"/>
+    </row>
+    <row r="756">
+      <c r="F756" s="7"/>
+    </row>
+    <row r="757">
+      <c r="F757" s="7"/>
+    </row>
+    <row r="758">
+      <c r="F758" s="7"/>
+    </row>
+    <row r="759">
+      <c r="F759" s="7"/>
+    </row>
+    <row r="760">
+      <c r="F760" s="7"/>
+    </row>
+    <row r="761">
+      <c r="F761" s="7"/>
+    </row>
+    <row r="762">
+      <c r="F762" s="7"/>
+    </row>
+    <row r="763">
+      <c r="F763" s="7"/>
+    </row>
+    <row r="764">
+      <c r="F764" s="7"/>
+    </row>
+    <row r="765">
+      <c r="F765" s="7"/>
+    </row>
+    <row r="766">
+      <c r="F766" s="7"/>
+    </row>
+    <row r="767">
+      <c r="F767" s="7"/>
+    </row>
+    <row r="768">
+      <c r="F768" s="7"/>
+    </row>
+    <row r="769">
+      <c r="F769" s="7"/>
+    </row>
+    <row r="770">
+      <c r="F770" s="7"/>
+    </row>
+    <row r="771">
+      <c r="F771" s="7"/>
+    </row>
+    <row r="772">
+      <c r="F772" s="7"/>
+    </row>
+    <row r="773">
+      <c r="F773" s="7"/>
+    </row>
+    <row r="774">
+      <c r="F774" s="7"/>
+    </row>
+    <row r="775">
+      <c r="F775" s="7"/>
+    </row>
+    <row r="776">
+      <c r="F776" s="7"/>
+    </row>
+    <row r="777">
+      <c r="F777" s="7"/>
+    </row>
+    <row r="778">
+      <c r="F778" s="7"/>
+    </row>
+    <row r="779">
+      <c r="F779" s="7"/>
+    </row>
+    <row r="780">
+      <c r="F780" s="7"/>
+    </row>
+    <row r="781">
+      <c r="F781" s="7"/>
+    </row>
+    <row r="782">
+      <c r="F782" s="7"/>
+    </row>
+    <row r="783">
+      <c r="F783" s="7"/>
+    </row>
+    <row r="784">
+      <c r="F784" s="7"/>
+    </row>
+    <row r="785">
+      <c r="F785" s="7"/>
+    </row>
+    <row r="786">
+      <c r="F786" s="7"/>
+    </row>
+    <row r="787">
+      <c r="F787" s="7"/>
+    </row>
+    <row r="788">
+      <c r="F788" s="7"/>
+    </row>
+    <row r="789">
+      <c r="F789" s="7"/>
+    </row>
+    <row r="790">
+      <c r="F790" s="7"/>
+    </row>
+    <row r="791">
+      <c r="F791" s="7"/>
+    </row>
+    <row r="792">
+      <c r="F792" s="7"/>
+    </row>
+    <row r="793">
+      <c r="F793" s="7"/>
+    </row>
+    <row r="794">
+      <c r="F794" s="7"/>
+    </row>
+    <row r="795">
+      <c r="F795" s="7"/>
+    </row>
+    <row r="796">
+      <c r="F796" s="7"/>
+    </row>
+    <row r="797">
+      <c r="F797" s="7"/>
+    </row>
+    <row r="798">
+      <c r="F798" s="7"/>
+    </row>
+    <row r="799">
+      <c r="F799" s="7"/>
+    </row>
+    <row r="800">
+      <c r="F800" s="7"/>
+    </row>
+    <row r="801">
+      <c r="F801" s="7"/>
+    </row>
+    <row r="802">
+      <c r="F802" s="7"/>
+    </row>
+    <row r="803">
+      <c r="F803" s="7"/>
+    </row>
+    <row r="804">
+      <c r="F804" s="7"/>
+    </row>
+    <row r="805">
+      <c r="F805" s="7"/>
+    </row>
+    <row r="806">
+      <c r="F806" s="7"/>
+    </row>
+    <row r="807">
+      <c r="F807" s="7"/>
+    </row>
+    <row r="808">
+      <c r="F808" s="7"/>
+    </row>
+    <row r="809">
+      <c r="F809" s="7"/>
+    </row>
+    <row r="810">
+      <c r="F810" s="7"/>
+    </row>
+    <row r="811">
+      <c r="F811" s="7"/>
+    </row>
+    <row r="812">
+      <c r="F812" s="7"/>
+    </row>
+    <row r="813">
+      <c r="F813" s="7"/>
+    </row>
+    <row r="814">
+      <c r="F814" s="7"/>
+    </row>
+    <row r="815">
+      <c r="F815" s="7"/>
+    </row>
+    <row r="816">
+      <c r="F816" s="7"/>
+    </row>
+    <row r="817">
+      <c r="F817" s="7"/>
+    </row>
+    <row r="818">
+      <c r="F818" s="7"/>
+    </row>
+    <row r="819">
+      <c r="F819" s="7"/>
+    </row>
+    <row r="820">
+      <c r="F820" s="7"/>
+    </row>
+    <row r="821">
+      <c r="F821" s="7"/>
+    </row>
+    <row r="822">
+      <c r="F822" s="7"/>
+    </row>
+    <row r="823">
+      <c r="F823" s="7"/>
+    </row>
+    <row r="824">
+      <c r="F824" s="7"/>
+    </row>
+    <row r="825">
+      <c r="F825" s="7"/>
+    </row>
+    <row r="826">
+      <c r="F826" s="7"/>
+    </row>
+    <row r="827">
+      <c r="F827" s="7"/>
+    </row>
+    <row r="828">
+      <c r="F828" s="7"/>
+    </row>
+    <row r="829">
+      <c r="F829" s="7"/>
+    </row>
+    <row r="830">
+      <c r="F830" s="7"/>
+    </row>
+    <row r="831">
+      <c r="F831" s="7"/>
+    </row>
+    <row r="832">
+      <c r="F832" s="7"/>
+    </row>
+    <row r="833">
+      <c r="F833" s="7"/>
+    </row>
+    <row r="834">
+      <c r="F834" s="7"/>
+    </row>
+    <row r="835">
+      <c r="F835" s="7"/>
+    </row>
+    <row r="836">
+      <c r="F836" s="7"/>
+    </row>
+    <row r="837">
+      <c r="F837" s="7"/>
+    </row>
+    <row r="838">
+      <c r="F838" s="7"/>
+    </row>
+    <row r="839">
+      <c r="F839" s="7"/>
+    </row>
+    <row r="840">
+      <c r="F840" s="7"/>
+    </row>
+    <row r="841">
+      <c r="F841" s="7"/>
+    </row>
+    <row r="842">
+      <c r="F842" s="7"/>
+    </row>
+    <row r="843">
+      <c r="F843" s="7"/>
+    </row>
+    <row r="844">
+      <c r="F844" s="7"/>
+    </row>
+    <row r="845">
+      <c r="F845" s="7"/>
+    </row>
+    <row r="846">
+      <c r="F846" s="7"/>
+    </row>
+    <row r="847">
+      <c r="F847" s="7"/>
+    </row>
+    <row r="848">
+      <c r="F848" s="7"/>
+    </row>
+    <row r="849">
+      <c r="F849" s="7"/>
+    </row>
+    <row r="850">
+      <c r="F850" s="7"/>
+    </row>
+    <row r="851">
+      <c r="F851" s="7"/>
+    </row>
+    <row r="852">
+      <c r="F852" s="7"/>
+    </row>
+    <row r="853">
+      <c r="F853" s="7"/>
+    </row>
+    <row r="854">
+      <c r="F854" s="7"/>
+    </row>
+    <row r="855">
+      <c r="F855" s="7"/>
+    </row>
+    <row r="856">
+      <c r="F856" s="7"/>
+    </row>
+    <row r="857">
+      <c r="F857" s="7"/>
+    </row>
+    <row r="858">
+      <c r="F858" s="7"/>
+    </row>
+    <row r="859">
+      <c r="F859" s="7"/>
+    </row>
+    <row r="860">
+      <c r="F860" s="7"/>
+    </row>
+    <row r="861">
+      <c r="F861" s="7"/>
+    </row>
+    <row r="862">
+      <c r="F862" s="7"/>
+    </row>
+    <row r="863">
+      <c r="F863" s="7"/>
+    </row>
+    <row r="864">
+      <c r="F864" s="7"/>
+    </row>
+    <row r="865">
+      <c r="F865" s="7"/>
+    </row>
+    <row r="866">
+      <c r="F866" s="7"/>
+    </row>
+    <row r="867">
+      <c r="F867" s="7"/>
+    </row>
+    <row r="868">
+      <c r="F868" s="7"/>
+    </row>
+    <row r="869">
+      <c r="F869" s="7"/>
+    </row>
+    <row r="870">
+      <c r="F870" s="7"/>
+    </row>
+    <row r="871">
+      <c r="F871" s="7"/>
+    </row>
+    <row r="872">
+      <c r="F872" s="7"/>
+    </row>
+    <row r="873">
+      <c r="F873" s="7"/>
+    </row>
+    <row r="874">
+      <c r="F874" s="7"/>
+    </row>
+    <row r="875">
+      <c r="F875" s="7"/>
+    </row>
+    <row r="876">
+      <c r="F876" s="7"/>
+    </row>
+    <row r="877">
+      <c r="F877" s="7"/>
+    </row>
+    <row r="878">
+      <c r="F878" s="7"/>
+    </row>
+    <row r="879">
+      <c r="F879" s="7"/>
+    </row>
+    <row r="880">
+      <c r="F880" s="7"/>
+    </row>
+    <row r="881">
+      <c r="F881" s="7"/>
+    </row>
+    <row r="882">
+      <c r="F882" s="7"/>
+    </row>
+    <row r="883">
+      <c r="F883" s="7"/>
+    </row>
+    <row r="884">
+      <c r="F884" s="7"/>
+    </row>
+    <row r="885">
+      <c r="F885" s="7"/>
+    </row>
+    <row r="886">
+      <c r="F886" s="7"/>
+    </row>
+    <row r="887">
+      <c r="F887" s="7"/>
+    </row>
+    <row r="888">
+      <c r="F888" s="7"/>
+    </row>
+    <row r="889">
+      <c r="F889" s="7"/>
+    </row>
+    <row r="890">
+      <c r="F890" s="7"/>
+    </row>
+    <row r="891">
+      <c r="F891" s="7"/>
+    </row>
+    <row r="892">
+      <c r="F892" s="7"/>
+    </row>
+    <row r="893">
+      <c r="F893" s="7"/>
+    </row>
+    <row r="894">
+      <c r="F894" s="7"/>
+    </row>
+    <row r="895">
+      <c r="F895" s="7"/>
+    </row>
+    <row r="896">
+      <c r="F896" s="7"/>
+    </row>
+    <row r="897">
+      <c r="F897" s="7"/>
+    </row>
+    <row r="898">
+      <c r="F898" s="7"/>
+    </row>
+    <row r="899">
+      <c r="F899" s="7"/>
+    </row>
+    <row r="900">
+      <c r="F900" s="7"/>
+    </row>
+    <row r="901">
+      <c r="F901" s="7"/>
+    </row>
+    <row r="902">
+      <c r="F902" s="7"/>
+    </row>
+    <row r="903">
+      <c r="F903" s="7"/>
+    </row>
+    <row r="904">
+      <c r="F904" s="7"/>
+    </row>
+    <row r="905">
+      <c r="F905" s="7"/>
+    </row>
+    <row r="906">
+      <c r="F906" s="7"/>
+    </row>
+    <row r="907">
+      <c r="F907" s="7"/>
+    </row>
+    <row r="908">
+      <c r="F908" s="7"/>
+    </row>
+    <row r="909">
+      <c r="F909" s="7"/>
+    </row>
+    <row r="910">
+      <c r="F910" s="7"/>
+    </row>
+    <row r="911">
+      <c r="F911" s="7"/>
+    </row>
+    <row r="912">
+      <c r="F912" s="7"/>
+    </row>
+    <row r="913">
+      <c r="F913" s="7"/>
+    </row>
+    <row r="914">
+      <c r="F914" s="7"/>
+    </row>
+    <row r="915">
+      <c r="F915" s="7"/>
+    </row>
+    <row r="916">
+      <c r="F916" s="7"/>
+    </row>
+    <row r="917">
+      <c r="F917" s="7"/>
+    </row>
+    <row r="918">
+      <c r="F918" s="7"/>
+    </row>
+    <row r="919">
+      <c r="F919" s="7"/>
+    </row>
+    <row r="920">
+      <c r="F920" s="7"/>
+    </row>
+    <row r="921">
+      <c r="F921" s="7"/>
+    </row>
+    <row r="922">
+      <c r="F922" s="7"/>
+    </row>
+    <row r="923">
+      <c r="F923" s="7"/>
+    </row>
+    <row r="924">
+      <c r="F924" s="7"/>
+    </row>
+    <row r="925">
+      <c r="F925" s="7"/>
+    </row>
+    <row r="926">
+      <c r="F926" s="7"/>
+    </row>
+    <row r="927">
+      <c r="F927" s="7"/>
+    </row>
+    <row r="928">
+      <c r="F928" s="7"/>
+    </row>
+    <row r="929">
+      <c r="F929" s="7"/>
+    </row>
+    <row r="930">
+      <c r="F930" s="7"/>
+    </row>
+    <row r="931">
+      <c r="F931" s="7"/>
+    </row>
+    <row r="932">
+      <c r="F932" s="7"/>
+    </row>
+    <row r="933">
+      <c r="F933" s="7"/>
+    </row>
+    <row r="934">
+      <c r="F934" s="7"/>
+    </row>
+    <row r="935">
+      <c r="F935" s="7"/>
+    </row>
+    <row r="936">
+      <c r="F936" s="7"/>
+    </row>
+    <row r="937">
+      <c r="F937" s="7"/>
+    </row>
+    <row r="938">
+      <c r="F938" s="7"/>
+    </row>
+    <row r="939">
+      <c r="F939" s="7"/>
+    </row>
+    <row r="940">
+      <c r="F940" s="7"/>
+    </row>
+    <row r="941">
+      <c r="F941" s="7"/>
+    </row>
+    <row r="942">
+      <c r="F942" s="7"/>
+    </row>
+    <row r="943">
+      <c r="F943" s="7"/>
+    </row>
+    <row r="944">
+      <c r="F944" s="7"/>
+    </row>
+    <row r="945">
+      <c r="F945" s="7"/>
+    </row>
+    <row r="946">
+      <c r="F946" s="7"/>
+    </row>
+    <row r="947">
+      <c r="F947" s="7"/>
+    </row>
+    <row r="948">
+      <c r="F948" s="7"/>
+    </row>
+    <row r="949">
+      <c r="F949" s="7"/>
+    </row>
+    <row r="950">
+      <c r="F950" s="7"/>
+    </row>
+    <row r="951">
+      <c r="F951" s="7"/>
+    </row>
+    <row r="952">
+      <c r="F952" s="7"/>
+    </row>
+    <row r="953">
+      <c r="F953" s="7"/>
+    </row>
+    <row r="954">
+      <c r="F954" s="7"/>
+    </row>
+    <row r="955">
+      <c r="F955" s="7"/>
+    </row>
+    <row r="956">
+      <c r="F956" s="7"/>
+    </row>
+    <row r="957">
+      <c r="F957" s="7"/>
+    </row>
+    <row r="958">
+      <c r="F958" s="7"/>
+    </row>
+    <row r="959">
+      <c r="F959" s="7"/>
+    </row>
+    <row r="960">
+      <c r="F960" s="7"/>
+    </row>
+    <row r="961">
+      <c r="F961" s="7"/>
+    </row>
+    <row r="962">
+      <c r="F962" s="7"/>
+    </row>
+    <row r="963">
+      <c r="F963" s="7"/>
+    </row>
+    <row r="964">
+      <c r="F964" s="7"/>
+    </row>
+    <row r="965">
+      <c r="F965" s="7"/>
+    </row>
+    <row r="966">
+      <c r="F966" s="7"/>
+    </row>
+    <row r="967">
+      <c r="F967" s="7"/>
+    </row>
+    <row r="968">
+      <c r="F968" s="7"/>
+    </row>
+    <row r="969">
+      <c r="F969" s="7"/>
+    </row>
+    <row r="970">
+      <c r="F970" s="7"/>
+    </row>
+    <row r="971">
+      <c r="F971" s="7"/>
+    </row>
+    <row r="972">
+      <c r="F972" s="7"/>
+    </row>
+    <row r="973">
+      <c r="F973" s="7"/>
+    </row>
+    <row r="974">
+      <c r="F974" s="7"/>
+    </row>
+    <row r="975">
+      <c r="F975" s="7"/>
+    </row>
+    <row r="976">
+      <c r="F976" s="7"/>
+    </row>
+    <row r="977">
+      <c r="F977" s="7"/>
+    </row>
+    <row r="978">
+      <c r="F978" s="7"/>
+    </row>
+    <row r="979">
+      <c r="F979" s="7"/>
+    </row>
+    <row r="980">
+      <c r="F980" s="7"/>
+    </row>
+    <row r="981">
+      <c r="F981" s="7"/>
+    </row>
+    <row r="982">
+      <c r="F982" s="7"/>
+    </row>
+    <row r="983">
+      <c r="F983" s="7"/>
+    </row>
+    <row r="984">
+      <c r="F984" s="7"/>
+    </row>
+    <row r="985">
+      <c r="F985" s="7"/>
+    </row>
+    <row r="986">
+      <c r="F986" s="7"/>
+    </row>
+    <row r="987">
+      <c r="F987" s="7"/>
+    </row>
+    <row r="988">
+      <c r="F988" s="7"/>
+    </row>
+    <row r="989">
+      <c r="F989" s="7"/>
+    </row>
+    <row r="990">
+      <c r="F990" s="7"/>
+    </row>
+    <row r="991">
+      <c r="F991" s="7"/>
+    </row>
+    <row r="992">
+      <c r="F992" s="7"/>
+    </row>
+    <row r="993">
+      <c r="F993" s="7"/>
+    </row>
+    <row r="994">
+      <c r="F994" s="7"/>
+    </row>
+    <row r="995">
+      <c r="F995" s="7"/>
+    </row>
+    <row r="996">
+      <c r="F996" s="7"/>
+    </row>
+    <row r="997">
+      <c r="F997" s="7"/>
+    </row>
+    <row r="998">
+      <c r="F998" s="7"/>
+    </row>
+    <row r="999">
+      <c r="F999" s="7"/>
+    </row>
+    <row r="1000">
+      <c r="F1000" s="7"/>
     </row>
   </sheetData>
   <drawing r:id="rId1"/>
@@ -20136,7 +23145,7 @@
       <c r="F1" s="1" t="s">
         <v>717</v>
       </c>
-      <c r="G1" s="13" t="s">
+      <c r="G1" s="14" t="s">
         <v>718</v>
       </c>
       <c r="H1" s="12"/>
@@ -20166,20 +23175,20 @@
         <v>Acorn Energy, Inc. (NASDAQCM:ACFN)</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>720</v>
-      </c>
-      <c r="C2" s="14" t="s">
-        <v>721</v>
-      </c>
-      <c r="D2" s="15" t="s">
-        <v>722</v>
+        <v>723</v>
+      </c>
+      <c r="C2" s="15" t="s">
+        <v>724</v>
+      </c>
+      <c r="D2" s="13" t="s">
+        <v>719</v>
       </c>
       <c r="E2" s="7"/>
-      <c r="F2" s="15">
+      <c r="F2" s="13">
         <v>22.52</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>723</v>
+        <v>725</v>
       </c>
     </row>
     <row r="3">
@@ -20188,20 +23197,20 @@
         <v>American Woodmark Corporation (NASDAQGS:AMWD)</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>720</v>
-      </c>
-      <c r="C3" s="14" t="s">
-        <v>721</v>
-      </c>
-      <c r="D3" s="15" t="s">
+        <v>723</v>
+      </c>
+      <c r="C3" s="15" t="s">
         <v>724</v>
       </c>
+      <c r="D3" s="13" t="s">
+        <v>722</v>
+      </c>
       <c r="E3" s="7"/>
-      <c r="F3" s="15">
+      <c r="F3" s="13">
         <v>40.75</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="4">
@@ -20210,20 +23219,20 @@
         <v>Artesian Resources Corporation (NASDAQGS:ARTN.A)</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>726</v>
-      </c>
-      <c r="C4" s="14" t="s">
-        <v>721</v>
-      </c>
-      <c r="D4" s="15" t="s">
         <v>727</v>
       </c>
+      <c r="C4" s="15" t="s">
+        <v>724</v>
+      </c>
+      <c r="D4" s="13" t="s">
+        <v>728</v>
+      </c>
       <c r="E4" s="7"/>
-      <c r="F4" s="15">
+      <c r="F4" s="13">
         <v>14.39</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>728</v>
+        <v>729</v>
       </c>
     </row>
     <row r="5">
@@ -20232,20 +23241,20 @@
         <v>Barrett Business Services, Inc. (NASDAQGS:BBSI)</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>726</v>
-      </c>
-      <c r="C5" s="14" t="s">
-        <v>721</v>
-      </c>
-      <c r="D5" s="15" t="s">
+        <v>727</v>
+      </c>
+      <c r="C5" s="15" t="s">
+        <v>724</v>
+      </c>
+      <c r="D5" s="13" t="s">
+        <v>730</v>
+      </c>
+      <c r="E5" s="7"/>
+      <c r="F5" s="13">
+        <v>20.85</v>
+      </c>
+      <c r="G5" s="5" t="s">
         <v>729</v>
-      </c>
-      <c r="E5" s="7"/>
-      <c r="F5" s="15">
-        <v>20.85</v>
-      </c>
-      <c r="G5" s="5" t="s">
-        <v>728</v>
       </c>
     </row>
     <row r="6">
@@ -20254,20 +23263,20 @@
         <v>Bassett Furniture Industries, Incorporated (NASDAQGS:BSET)</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>720</v>
-      </c>
-      <c r="C6" s="14" t="s">
-        <v>721</v>
-      </c>
-      <c r="D6" s="15" t="s">
+        <v>723</v>
+      </c>
+      <c r="C6" s="15" t="s">
         <v>724</v>
       </c>
+      <c r="D6" s="13" t="s">
+        <v>722</v>
+      </c>
       <c r="E6" s="7"/>
-      <c r="F6" s="15">
+      <c r="F6" s="13">
         <v>23.42</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="7">
@@ -20276,20 +23285,20 @@
         <v>BJ's Restaurants, Inc. (NASDAQGS:BJRI)</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>720</v>
-      </c>
-      <c r="C7" s="14" t="s">
-        <v>721</v>
-      </c>
-      <c r="D7" s="15" t="s">
-        <v>730</v>
+        <v>723</v>
+      </c>
+      <c r="C7" s="15" t="s">
+        <v>724</v>
+      </c>
+      <c r="D7" s="13" t="s">
+        <v>731</v>
       </c>
       <c r="E7" s="7"/>
-      <c r="F7" s="15">
+      <c r="F7" s="13">
         <v>21.63</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>731</v>
+        <v>732</v>
       </c>
     </row>
     <row r="8">
@@ -20298,22 +23307,22 @@
         <v>Build-A-Bear Workshop, Inc. (NYSE:BBW)</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>720</v>
-      </c>
-      <c r="C8" s="14" t="s">
-        <v>721</v>
-      </c>
-      <c r="D8" s="15" t="s">
+        <v>723</v>
+      </c>
+      <c r="C8" s="15" t="s">
+        <v>724</v>
+      </c>
+      <c r="D8" s="13" t="s">
+        <v>733</v>
+      </c>
+      <c r="E8" s="13" t="s">
+        <v>734</v>
+      </c>
+      <c r="F8" s="13">
+        <v>8.38</v>
+      </c>
+      <c r="G8" s="5" t="s">
         <v>732</v>
-      </c>
-      <c r="E8" s="15" t="s">
-        <v>733</v>
-      </c>
-      <c r="F8" s="15">
-        <v>8.38</v>
-      </c>
-      <c r="G8" s="5" t="s">
-        <v>731</v>
       </c>
     </row>
     <row r="9">
@@ -20322,20 +23331,20 @@
         <v>Carriage Services, Inc. (NYSE:CSV)</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>726</v>
-      </c>
-      <c r="C9" s="14" t="s">
-        <v>721</v>
-      </c>
-      <c r="D9" s="15" t="s">
+        <v>727</v>
+      </c>
+      <c r="C9" s="15" t="s">
+        <v>724</v>
+      </c>
+      <c r="D9" s="13" t="s">
+        <v>730</v>
+      </c>
+      <c r="E9" s="7"/>
+      <c r="F9" s="13">
+        <v>14.73</v>
+      </c>
+      <c r="G9" s="5" t="s">
         <v>729</v>
-      </c>
-      <c r="E9" s="7"/>
-      <c r="F9" s="15">
-        <v>14.73</v>
-      </c>
-      <c r="G9" s="5" t="s">
-        <v>728</v>
       </c>
     </row>
     <row r="10">
@@ -20345,15 +23354,15 @@
       </c>
       <c r="B10" s="6"/>
       <c r="C10" s="7"/>
-      <c r="D10" s="15" t="s">
-        <v>730</v>
+      <c r="D10" s="13" t="s">
+        <v>731</v>
       </c>
       <c r="E10" s="7"/>
-      <c r="F10" s="15" t="s">
-        <v>734</v>
+      <c r="F10" s="13" t="s">
+        <v>720</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>731</v>
+        <v>732</v>
       </c>
     </row>
     <row r="11">
@@ -20363,15 +23372,15 @@
       </c>
       <c r="B11" s="6"/>
       <c r="C11" s="7"/>
-      <c r="D11" s="15" t="s">
-        <v>724</v>
+      <c r="D11" s="13" t="s">
+        <v>722</v>
       </c>
       <c r="E11" s="7"/>
-      <c r="F11" s="15">
+      <c r="F11" s="13">
         <v>12.91</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>723</v>
+        <v>725</v>
       </c>
     </row>
     <row r="12">
@@ -20381,15 +23390,15 @@
       </c>
       <c r="B12" s="6"/>
       <c r="C12" s="7"/>
-      <c r="D12" s="15" t="s">
+      <c r="D12" s="13" t="s">
         <v>735</v>
       </c>
       <c r="E12" s="7"/>
-      <c r="F12" s="15">
+      <c r="F12" s="13">
         <v>14.82</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>728</v>
+        <v>729</v>
       </c>
     </row>
     <row r="13">
@@ -20399,11 +23408,11 @@
       </c>
       <c r="B13" s="6"/>
       <c r="C13" s="7"/>
-      <c r="D13" s="15" t="s">
-        <v>722</v>
+      <c r="D13" s="13" t="s">
+        <v>719</v>
       </c>
       <c r="E13" s="7"/>
-      <c r="F13" s="15">
+      <c r="F13" s="13">
         <v>51.98</v>
       </c>
       <c r="G13" s="5" t="s">
@@ -20417,15 +23426,15 @@
       </c>
       <c r="B14" s="6"/>
       <c r="C14" s="7"/>
-      <c r="D14" s="15" t="s">
-        <v>730</v>
+      <c r="D14" s="13" t="s">
+        <v>731</v>
       </c>
       <c r="E14" s="7"/>
-      <c r="F14" s="15">
+      <c r="F14" s="13">
         <v>319.5</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>731</v>
+        <v>732</v>
       </c>
     </row>
     <row r="15">
@@ -20435,15 +23444,15 @@
       </c>
       <c r="B15" s="6"/>
       <c r="C15" s="7"/>
-      <c r="D15" s="15" t="s">
-        <v>730</v>
+      <c r="D15" s="13" t="s">
+        <v>731</v>
       </c>
       <c r="E15" s="7"/>
-      <c r="F15" s="15">
+      <c r="F15" s="13">
         <v>27.3</v>
       </c>
       <c r="G15" s="5" t="s">
-        <v>731</v>
+        <v>732</v>
       </c>
     </row>
     <row r="16">
@@ -20453,15 +23462,15 @@
       </c>
       <c r="B16" s="6"/>
       <c r="C16" s="7"/>
-      <c r="D16" s="15" t="s">
+      <c r="D16" s="13" t="s">
         <v>737</v>
       </c>
       <c r="E16" s="7"/>
-      <c r="F16" s="15">
+      <c r="F16" s="13">
         <v>19.78</v>
       </c>
       <c r="G16" s="5" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="17">
@@ -20471,15 +23480,15 @@
       </c>
       <c r="B17" s="6"/>
       <c r="C17" s="7"/>
-      <c r="D17" s="15" t="s">
-        <v>730</v>
+      <c r="D17" s="13" t="s">
+        <v>731</v>
       </c>
       <c r="E17" s="7"/>
-      <c r="F17" s="15">
+      <c r="F17" s="13">
         <v>15.05</v>
       </c>
       <c r="G17" s="5" t="s">
-        <v>731</v>
+        <v>732</v>
       </c>
     </row>
     <row r="18">
@@ -20489,11 +23498,11 @@
       </c>
       <c r="B18" s="6"/>
       <c r="C18" s="7"/>
-      <c r="D18" s="15" t="s">
+      <c r="D18" s="13" t="s">
         <v>737</v>
       </c>
       <c r="E18" s="7"/>
-      <c r="F18" s="15">
+      <c r="F18" s="13">
         <v>95.88</v>
       </c>
       <c r="G18" s="5" t="s">
@@ -20507,15 +23516,15 @@
       </c>
       <c r="B19" s="6"/>
       <c r="C19" s="7"/>
-      <c r="D19" s="15" t="s">
-        <v>729</v>
+      <c r="D19" s="13" t="s">
+        <v>730</v>
       </c>
       <c r="E19" s="7"/>
-      <c r="F19" s="15" t="s">
-        <v>734</v>
+      <c r="F19" s="13" t="s">
+        <v>720</v>
       </c>
       <c r="G19" s="5" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="20">
@@ -20525,11 +23534,11 @@
       </c>
       <c r="B20" s="6"/>
       <c r="C20" s="7"/>
-      <c r="D20" s="15" t="s">
+      <c r="D20" s="13" t="s">
         <v>737</v>
       </c>
       <c r="E20" s="7"/>
-      <c r="F20" s="15">
+      <c r="F20" s="13">
         <v>21.62</v>
       </c>
       <c r="G20" s="5" t="s">
@@ -20543,15 +23552,15 @@
       </c>
       <c r="B21" s="6"/>
       <c r="C21" s="7"/>
-      <c r="D21" s="15" t="s">
+      <c r="D21" s="13" t="s">
         <v>735</v>
       </c>
       <c r="E21" s="7"/>
-      <c r="F21" s="15">
+      <c r="F21" s="13">
         <v>27.47</v>
       </c>
       <c r="G21" s="5" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="22">
@@ -20561,15 +23570,15 @@
       </c>
       <c r="B22" s="6"/>
       <c r="C22" s="7"/>
-      <c r="D22" s="15" t="s">
-        <v>724</v>
+      <c r="D22" s="13" t="s">
+        <v>722</v>
       </c>
       <c r="E22" s="7"/>
-      <c r="F22" s="15">
+      <c r="F22" s="13">
         <v>13.06</v>
       </c>
       <c r="G22" s="5" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="23">
@@ -20579,11 +23588,11 @@
       </c>
       <c r="B23" s="6"/>
       <c r="C23" s="7"/>
-      <c r="D23" s="15" t="s">
+      <c r="D23" s="13" t="s">
         <v>740</v>
       </c>
       <c r="E23" s="7"/>
-      <c r="F23" s="15">
+      <c r="F23" s="13">
         <v>17.46</v>
       </c>
       <c r="G23" s="5" t="s">
@@ -20597,11 +23606,11 @@
       </c>
       <c r="B24" s="6"/>
       <c r="C24" s="7"/>
-      <c r="D24" s="15" t="s">
-        <v>724</v>
+      <c r="D24" s="13" t="s">
+        <v>722</v>
       </c>
       <c r="E24" s="7"/>
-      <c r="F24" s="15">
+      <c r="F24" s="13">
         <v>15.48</v>
       </c>
       <c r="G24" s="5" t="s">
@@ -20615,15 +23624,15 @@
       </c>
       <c r="B25" s="6"/>
       <c r="C25" s="7"/>
-      <c r="D25" s="15" t="s">
+      <c r="D25" s="13" t="s">
         <v>742</v>
       </c>
       <c r="E25" s="7"/>
-      <c r="F25" s="15">
+      <c r="F25" s="13">
         <v>15.54</v>
       </c>
       <c r="G25" s="5" t="s">
-        <v>728</v>
+        <v>729</v>
       </c>
     </row>
     <row r="26">
@@ -20633,15 +23642,15 @@
       </c>
       <c r="B26" s="6"/>
       <c r="C26" s="7"/>
-      <c r="D26" s="15" t="s">
+      <c r="D26" s="13" t="s">
         <v>737</v>
       </c>
       <c r="E26" s="7"/>
-      <c r="F26" s="15" t="s">
-        <v>734</v>
+      <c r="F26" s="13" t="s">
+        <v>720</v>
       </c>
       <c r="G26" s="5" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="27">
@@ -20651,15 +23660,15 @@
       </c>
       <c r="B27" s="6"/>
       <c r="C27" s="7"/>
-      <c r="D27" s="15" t="s">
+      <c r="D27" s="13" t="s">
         <v>737</v>
       </c>
       <c r="E27" s="7"/>
-      <c r="F27" s="15">
+      <c r="F27" s="13">
         <v>10.66</v>
       </c>
       <c r="G27" s="5" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="28">
@@ -20669,11 +23678,11 @@
       </c>
       <c r="B28" s="6"/>
       <c r="C28" s="7"/>
-      <c r="D28" s="15" t="s">
+      <c r="D28" s="13" t="s">
         <v>740</v>
       </c>
       <c r="E28" s="7"/>
-      <c r="F28" s="15">
+      <c r="F28" s="13">
         <v>462.4</v>
       </c>
       <c r="G28" s="5" t="s">
@@ -20687,15 +23696,15 @@
       </c>
       <c r="B29" s="6"/>
       <c r="C29" s="7"/>
-      <c r="D29" s="15" t="s">
-        <v>730</v>
+      <c r="D29" s="13" t="s">
+        <v>731</v>
       </c>
       <c r="E29" s="7"/>
-      <c r="F29" s="15" t="s">
-        <v>734</v>
+      <c r="F29" s="13" t="s">
+        <v>720</v>
       </c>
       <c r="G29" s="5" t="s">
-        <v>731</v>
+        <v>732</v>
       </c>
     </row>
     <row r="30">
@@ -20705,11 +23714,11 @@
       </c>
       <c r="B30" s="6"/>
       <c r="C30" s="7"/>
-      <c r="D30" s="15" t="s">
+      <c r="D30" s="13" t="s">
         <v>735</v>
       </c>
       <c r="E30" s="7"/>
-      <c r="F30" s="15">
+      <c r="F30" s="13">
         <v>22.56</v>
       </c>
       <c r="G30" s="5" t="s">
@@ -20723,15 +23732,15 @@
       </c>
       <c r="B31" s="6"/>
       <c r="C31" s="7"/>
-      <c r="D31" s="15" t="s">
+      <c r="D31" s="13" t="s">
         <v>737</v>
       </c>
       <c r="E31" s="7"/>
-      <c r="F31" s="15">
+      <c r="F31" s="13">
         <v>48.74</v>
       </c>
       <c r="G31" s="5" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="32">
@@ -20741,11 +23750,11 @@
       </c>
       <c r="B32" s="6"/>
       <c r="C32" s="7"/>
-      <c r="D32" s="15" t="s">
+      <c r="D32" s="13" t="s">
         <v>740</v>
       </c>
       <c r="E32" s="7"/>
-      <c r="F32" s="15">
+      <c r="F32" s="13">
         <v>30.29</v>
       </c>
       <c r="G32" s="5" t="s">
@@ -20759,15 +23768,15 @@
       </c>
       <c r="B33" s="6"/>
       <c r="C33" s="7"/>
-      <c r="D33" s="15" t="s">
-        <v>727</v>
+      <c r="D33" s="13" t="s">
+        <v>728</v>
       </c>
       <c r="E33" s="7"/>
-      <c r="F33" s="15">
+      <c r="F33" s="13">
         <v>92.25</v>
       </c>
       <c r="G33" s="5" t="s">
-        <v>728</v>
+        <v>729</v>
       </c>
     </row>
     <row r="34">
@@ -20777,15 +23786,15 @@
       </c>
       <c r="B34" s="6"/>
       <c r="C34" s="7"/>
-      <c r="D34" s="15" t="s">
+      <c r="D34" s="13" t="s">
         <v>743</v>
       </c>
       <c r="E34" s="7"/>
-      <c r="F34" s="15">
+      <c r="F34" s="13">
         <v>129.77</v>
       </c>
       <c r="G34" s="5" t="s">
-        <v>731</v>
+        <v>732</v>
       </c>
     </row>
     <row r="35">
@@ -20795,15 +23804,15 @@
       </c>
       <c r="B35" s="6"/>
       <c r="C35" s="7"/>
-      <c r="D35" s="15" t="s">
-        <v>730</v>
+      <c r="D35" s="13" t="s">
+        <v>731</v>
       </c>
       <c r="E35" s="7"/>
-      <c r="F35" s="15">
+      <c r="F35" s="13">
         <v>7.71</v>
       </c>
       <c r="G35" s="5" t="s">
-        <v>731</v>
+        <v>732</v>
       </c>
     </row>
     <row r="36">
@@ -20813,15 +23822,15 @@
       </c>
       <c r="B36" s="6"/>
       <c r="C36" s="7"/>
-      <c r="D36" s="15" t="s">
-        <v>724</v>
+      <c r="D36" s="13" t="s">
+        <v>722</v>
       </c>
       <c r="E36" s="7"/>
-      <c r="F36" s="15">
+      <c r="F36" s="13">
         <v>9.54</v>
       </c>
       <c r="G36" s="5" t="s">
-        <v>728</v>
+        <v>729</v>
       </c>
     </row>
     <row r="37">
@@ -20831,15 +23840,15 @@
       </c>
       <c r="B37" s="6"/>
       <c r="C37" s="7"/>
-      <c r="D37" s="15" t="s">
-        <v>732</v>
+      <c r="D37" s="13" t="s">
+        <v>733</v>
       </c>
       <c r="E37" s="7"/>
-      <c r="F37" s="15">
+      <c r="F37" s="13">
         <v>9.49</v>
       </c>
       <c r="G37" s="5" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="38">
@@ -20849,15 +23858,15 @@
       </c>
       <c r="B38" s="6"/>
       <c r="C38" s="7"/>
-      <c r="D38" s="15" t="s">
-        <v>724</v>
+      <c r="D38" s="13" t="s">
+        <v>722</v>
       </c>
       <c r="E38" s="7"/>
-      <c r="F38" s="15" t="s">
-        <v>734</v>
+      <c r="F38" s="13" t="s">
+        <v>720</v>
       </c>
       <c r="G38" s="5" t="s">
-        <v>728</v>
+        <v>729</v>
       </c>
     </row>
     <row r="39">
@@ -20867,15 +23876,15 @@
       </c>
       <c r="B39" s="6"/>
       <c r="C39" s="7"/>
-      <c r="D39" s="15" t="s">
+      <c r="D39" s="13" t="s">
         <v>737</v>
       </c>
       <c r="E39" s="7"/>
-      <c r="F39" s="15" t="s">
-        <v>734</v>
+      <c r="F39" s="13" t="s">
+        <v>720</v>
       </c>
       <c r="G39" s="5" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
     </row>
     <row r="40">

</xml_diff>

<commit_message>
Add Cricut qualitative assessment
</commit_message>
<xml_diff>
--- a/public/research/initial-screenings/Initial Screening (Under 1B MC, Over $0 NI).xlsx
+++ b/public/research/initial-screenings/Initial Screening (Under 1B MC, Over $0 NI).xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1587" uniqueCount="744">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1591" uniqueCount="744">
   <si>
     <t>Entity Name</t>
   </si>
@@ -23307,7 +23307,7 @@
         <v>Build-A-Bear Workshop, Inc. (NYSE:BBW)</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>723</v>
+        <v>727</v>
       </c>
       <c r="C8" s="15" t="s">
         <v>724</v>
@@ -23352,8 +23352,12 @@
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Cracker Barrel Old Country Store, Inc. (NASDAQGS:CBRL)")</f>
         <v>Cracker Barrel Old Country Store, Inc. (NASDAQGS:CBRL)</v>
       </c>
-      <c r="B10" s="6"/>
-      <c r="C10" s="7"/>
+      <c r="B10" s="5" t="s">
+        <v>723</v>
+      </c>
+      <c r="C10" s="15" t="s">
+        <v>724</v>
+      </c>
       <c r="D10" s="13" t="s">
         <v>731</v>
       </c>
@@ -23370,8 +23374,12 @@
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Cricut, Inc. (NASDAQGS:CRCT)")</f>
         <v>Cricut, Inc. (NASDAQGS:CRCT)</v>
       </c>
-      <c r="B11" s="6"/>
-      <c r="C11" s="7"/>
+      <c r="B11" s="5" t="s">
+        <v>727</v>
+      </c>
+      <c r="C11" s="15" t="s">
+        <v>724</v>
+      </c>
       <c r="D11" s="13" t="s">
         <v>722</v>
       </c>
@@ -30628,7 +30636,9 @@
     <hyperlink r:id="rId6" ref="C7"/>
     <hyperlink r:id="rId7" ref="C8"/>
     <hyperlink r:id="rId8" ref="C9"/>
+    <hyperlink r:id="rId9" ref="C10"/>
+    <hyperlink r:id="rId10" ref="C11"/>
   </hyperlinks>
-  <drawing r:id="rId9"/>
+  <drawing r:id="rId11"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update research documents and qualitative assessments
</commit_message>
<xml_diff>
--- a/public/research/initial-screenings/Initial Screening (Under 1B MC, Over $0 NI).xlsx
+++ b/public/research/initial-screenings/Initial Screening (Under 1B MC, Over $0 NI).xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2005" uniqueCount="748">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2023" uniqueCount="750">
   <si>
     <t>Entity Name</t>
   </si>
@@ -2222,6 +2222,9 @@
     <t>Restaurants</t>
   </si>
   <si>
+    <t>N/A</t>
+  </si>
+  <si>
     <t>Retail / Restaurant / Unit Economics Template</t>
   </si>
   <si>
@@ -2231,15 +2234,15 @@
     <t>Watchlist</t>
   </si>
   <si>
-    <t>N/M</t>
-  </si>
-  <si>
     <t>Energy</t>
   </si>
   <si>
     <t>Holding Company / Sum-of-the-Parts Template</t>
   </si>
   <si>
+    <t>Gaming &amp; Entertainment</t>
+  </si>
+  <si>
     <t>Industrials</t>
   </si>
   <si>
@@ -2258,10 +2261,13 @@
     <t>Healthcare</t>
   </si>
   <si>
-    <t>Gaming &amp; Entertainment</t>
-  </si>
-  <si>
     <t>Cigar Butt</t>
+  </si>
+  <si>
+    <t>Declining  Cigar-Butt  Runoff Cash Flow Template</t>
+  </si>
+  <si>
+    <t>Education</t>
   </si>
 </sst>
 </file>
@@ -25069,7 +25075,7 @@
       </c>
       <c r="E2" s="7"/>
       <c r="F2" s="10">
-        <v>22.52</v>
+        <v>20.7</v>
       </c>
       <c r="G2" s="5" t="s">
         <v>725</v>
@@ -25113,7 +25119,7 @@
       </c>
       <c r="E4" s="7"/>
       <c r="F4" s="10">
-        <v>14.39</v>
+        <v>14.65</v>
       </c>
       <c r="G4" s="5" t="s">
         <v>730</v>
@@ -25137,7 +25143,7 @@
         <v>732</v>
       </c>
       <c r="F5" s="10">
-        <v>20.85</v>
+        <v>20.37</v>
       </c>
       <c r="G5" s="5" t="s">
         <v>730</v>
@@ -25159,7 +25165,7 @@
       </c>
       <c r="E6" s="7"/>
       <c r="F6" s="10">
-        <v>23.42</v>
+        <v>22.94</v>
       </c>
       <c r="G6" s="5" t="s">
         <v>727</v>
@@ -25180,11 +25186,11 @@
         <v>733</v>
       </c>
       <c r="E7" s="7"/>
-      <c r="F7" s="10">
-        <v>21.63</v>
+      <c r="F7" s="10" t="s">
+        <v>734</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>734</v>
+        <v>735</v>
       </c>
     </row>
     <row r="8">
@@ -25199,16 +25205,16 @@
         <v>723</v>
       </c>
       <c r="D8" s="10" t="s">
+        <v>736</v>
+      </c>
+      <c r="E8" s="10" t="s">
+        <v>737</v>
+      </c>
+      <c r="F8" s="10">
+        <v>7.83</v>
+      </c>
+      <c r="G8" s="5" t="s">
         <v>735</v>
-      </c>
-      <c r="E8" s="10" t="s">
-        <v>736</v>
-      </c>
-      <c r="F8" s="10">
-        <v>8.38</v>
-      </c>
-      <c r="G8" s="5" t="s">
-        <v>734</v>
       </c>
     </row>
     <row r="9">
@@ -25227,7 +25233,7 @@
       </c>
       <c r="E9" s="7"/>
       <c r="F9" s="10">
-        <v>14.73</v>
+        <v>13.65</v>
       </c>
       <c r="G9" s="5" t="s">
         <v>730</v>
@@ -25248,11 +25254,11 @@
         <v>733</v>
       </c>
       <c r="E10" s="7"/>
-      <c r="F10" s="10" t="s">
-        <v>737</v>
+      <c r="F10" s="10">
+        <v>-176.53</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>734</v>
+        <v>735</v>
       </c>
     </row>
     <row r="11">
@@ -25271,7 +25277,7 @@
       </c>
       <c r="E11" s="7"/>
       <c r="F11" s="10">
-        <v>12.91</v>
+        <v>12.18</v>
       </c>
       <c r="G11" s="5" t="s">
         <v>725</v>
@@ -25289,7 +25295,7 @@
       </c>
       <c r="E12" s="7"/>
       <c r="F12" s="10">
-        <v>14.82</v>
+        <v>14.93</v>
       </c>
       <c r="G12" s="5" t="s">
         <v>730</v>
@@ -25307,7 +25313,7 @@
       </c>
       <c r="E13" s="7"/>
       <c r="F13" s="10">
-        <v>51.98</v>
+        <v>51.22</v>
       </c>
       <c r="G13" s="5" t="s">
         <v>739</v>
@@ -25321,14 +25327,14 @@
       <c r="B14" s="6"/>
       <c r="C14" s="7"/>
       <c r="D14" s="10" t="s">
-        <v>733</v>
+        <v>740</v>
       </c>
       <c r="E14" s="7"/>
       <c r="F14" s="10">
-        <v>319.5</v>
+        <v>280.0</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>734</v>
+        <v>735</v>
       </c>
     </row>
     <row r="15">
@@ -25343,10 +25349,10 @@
       </c>
       <c r="E15" s="7"/>
       <c r="F15" s="10">
-        <v>27.3</v>
+        <v>25.6</v>
       </c>
       <c r="G15" s="5" t="s">
-        <v>734</v>
+        <v>735</v>
       </c>
     </row>
     <row r="16">
@@ -25357,11 +25363,11 @@
       <c r="B16" s="6"/>
       <c r="C16" s="7"/>
       <c r="D16" s="10" t="s">
-        <v>740</v>
+        <v>741</v>
       </c>
       <c r="E16" s="7"/>
       <c r="F16" s="10">
-        <v>19.78</v>
+        <v>20.03</v>
       </c>
       <c r="G16" s="5" t="s">
         <v>727</v>
@@ -25379,10 +25385,10 @@
       </c>
       <c r="E17" s="7"/>
       <c r="F17" s="10">
-        <v>15.05</v>
+        <v>14.1</v>
       </c>
       <c r="G17" s="5" t="s">
-        <v>734</v>
+        <v>735</v>
       </c>
     </row>
     <row r="18">
@@ -25393,14 +25399,14 @@
       <c r="B18" s="6"/>
       <c r="C18" s="7"/>
       <c r="D18" s="10" t="s">
-        <v>740</v>
+        <v>741</v>
       </c>
       <c r="E18" s="7"/>
       <c r="F18" s="10">
-        <v>95.88</v>
+        <v>95.75</v>
       </c>
       <c r="G18" s="5" t="s">
-        <v>741</v>
+        <v>742</v>
       </c>
     </row>
     <row r="19">
@@ -25414,8 +25420,8 @@
         <v>731</v>
       </c>
       <c r="E19" s="7"/>
-      <c r="F19" s="10" t="s">
-        <v>737</v>
+      <c r="F19" s="10">
+        <v>-26.16</v>
       </c>
       <c r="G19" s="5" t="s">
         <v>727</v>
@@ -25429,14 +25435,14 @@
       <c r="B20" s="6"/>
       <c r="C20" s="7"/>
       <c r="D20" s="10" t="s">
-        <v>740</v>
+        <v>741</v>
       </c>
       <c r="E20" s="7"/>
       <c r="F20" s="10">
-        <v>21.62</v>
+        <v>21.65</v>
       </c>
       <c r="G20" s="5" t="s">
-        <v>742</v>
+        <v>743</v>
       </c>
     </row>
     <row r="21">
@@ -25451,7 +25457,7 @@
       </c>
       <c r="E21" s="7"/>
       <c r="F21" s="10">
-        <v>27.47</v>
+        <v>27.13</v>
       </c>
       <c r="G21" s="5" t="s">
         <v>727</v>
@@ -25469,7 +25475,7 @@
       </c>
       <c r="E22" s="7"/>
       <c r="F22" s="10">
-        <v>13.06</v>
+        <v>13.08</v>
       </c>
       <c r="G22" s="5" t="s">
         <v>727</v>
@@ -25483,14 +25489,14 @@
       <c r="B23" s="6"/>
       <c r="C23" s="7"/>
       <c r="D23" s="10" t="s">
-        <v>743</v>
+        <v>744</v>
       </c>
       <c r="E23" s="7"/>
       <c r="F23" s="10">
-        <v>17.46</v>
+        <v>17.51</v>
       </c>
       <c r="G23" s="5" t="s">
-        <v>744</v>
+        <v>745</v>
       </c>
     </row>
     <row r="24">
@@ -25505,10 +25511,10 @@
       </c>
       <c r="E24" s="7"/>
       <c r="F24" s="10">
-        <v>15.48</v>
+        <v>15.42</v>
       </c>
       <c r="G24" s="5" t="s">
-        <v>742</v>
+        <v>743</v>
       </c>
     </row>
     <row r="25">
@@ -25519,11 +25525,11 @@
       <c r="B25" s="6"/>
       <c r="C25" s="7"/>
       <c r="D25" s="10" t="s">
-        <v>745</v>
+        <v>746</v>
       </c>
       <c r="E25" s="7"/>
-      <c r="F25" s="10">
-        <v>15.54</v>
+      <c r="F25" s="10" t="s">
+        <v>734</v>
       </c>
       <c r="G25" s="5" t="s">
         <v>730</v>
@@ -25537,11 +25543,11 @@
       <c r="B26" s="6"/>
       <c r="C26" s="7"/>
       <c r="D26" s="10" t="s">
-        <v>740</v>
+        <v>726</v>
       </c>
       <c r="E26" s="7"/>
-      <c r="F26" s="10" t="s">
-        <v>737</v>
+      <c r="F26" s="10">
+        <v>-2.43</v>
       </c>
       <c r="G26" s="5" t="s">
         <v>727</v>
@@ -25555,11 +25561,11 @@
       <c r="B27" s="6"/>
       <c r="C27" s="7"/>
       <c r="D27" s="10" t="s">
-        <v>740</v>
+        <v>741</v>
       </c>
       <c r="E27" s="7"/>
       <c r="F27" s="10">
-        <v>10.66</v>
+        <v>10.94</v>
       </c>
       <c r="G27" s="5" t="s">
         <v>727</v>
@@ -25573,14 +25579,14 @@
       <c r="B28" s="6"/>
       <c r="C28" s="7"/>
       <c r="D28" s="10" t="s">
-        <v>743</v>
+        <v>744</v>
       </c>
       <c r="E28" s="7"/>
       <c r="F28" s="10">
-        <v>462.4</v>
+        <v>470.8</v>
       </c>
       <c r="G28" s="5" t="s">
-        <v>744</v>
+        <v>745</v>
       </c>
     </row>
     <row r="29">
@@ -25594,11 +25600,11 @@
         <v>733</v>
       </c>
       <c r="E29" s="7"/>
-      <c r="F29" s="10" t="s">
-        <v>737</v>
+      <c r="F29" s="10">
+        <v>-2.56</v>
       </c>
       <c r="G29" s="5" t="s">
-        <v>734</v>
+        <v>735</v>
       </c>
     </row>
     <row r="30">
@@ -25613,7 +25619,7 @@
       </c>
       <c r="E30" s="7"/>
       <c r="F30" s="10">
-        <v>22.56</v>
+        <v>22.89</v>
       </c>
       <c r="G30" s="5" t="s">
         <v>739</v>
@@ -25627,11 +25633,11 @@
       <c r="B31" s="6"/>
       <c r="C31" s="7"/>
       <c r="D31" s="10" t="s">
-        <v>740</v>
+        <v>741</v>
       </c>
       <c r="E31" s="7"/>
       <c r="F31" s="10">
-        <v>48.74</v>
+        <v>49.66</v>
       </c>
       <c r="G31" s="5" t="s">
         <v>727</v>
@@ -25645,14 +25651,14 @@
       <c r="B32" s="6"/>
       <c r="C32" s="7"/>
       <c r="D32" s="10" t="s">
-        <v>743</v>
+        <v>744</v>
       </c>
       <c r="E32" s="7"/>
       <c r="F32" s="10">
-        <v>30.29</v>
+        <v>29.82</v>
       </c>
       <c r="G32" s="5" t="s">
-        <v>744</v>
+        <v>745</v>
       </c>
     </row>
     <row r="33">
@@ -25667,7 +25673,7 @@
       </c>
       <c r="E33" s="7"/>
       <c r="F33" s="10">
-        <v>92.25</v>
+        <v>90.5</v>
       </c>
       <c r="G33" s="5" t="s">
         <v>730</v>
@@ -25681,14 +25687,14 @@
       <c r="B34" s="6"/>
       <c r="C34" s="7"/>
       <c r="D34" s="10" t="s">
-        <v>746</v>
+        <v>740</v>
       </c>
       <c r="E34" s="7"/>
       <c r="F34" s="10">
         <v>129.77</v>
       </c>
       <c r="G34" s="5" t="s">
-        <v>734</v>
+        <v>735</v>
       </c>
     </row>
     <row r="35">
@@ -25709,10 +25715,10 @@
         <v>747</v>
       </c>
       <c r="F35" s="10">
-        <v>7.71</v>
+        <v>7.65</v>
       </c>
       <c r="G35" s="5" t="s">
-        <v>734</v>
+        <v>735</v>
       </c>
     </row>
     <row r="36">
@@ -25727,7 +25733,7 @@
       </c>
       <c r="E36" s="7"/>
       <c r="F36" s="10">
-        <v>9.54</v>
+        <v>9.35</v>
       </c>
       <c r="G36" s="5" t="s">
         <v>730</v>
@@ -25741,11 +25747,11 @@
       <c r="B37" s="6"/>
       <c r="C37" s="7"/>
       <c r="D37" s="10" t="s">
-        <v>735</v>
+        <v>736</v>
       </c>
       <c r="E37" s="7"/>
       <c r="F37" s="10">
-        <v>9.49</v>
+        <v>9.43</v>
       </c>
       <c r="G37" s="5" t="s">
         <v>727</v>
@@ -25756,17 +25762,21 @@
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Helen of Troy Limited (NASDAQGS:HELE)")</f>
         <v>Helen of Troy Limited (NASDAQGS:HELE)</v>
       </c>
-      <c r="B38" s="6"/>
-      <c r="C38" s="7"/>
+      <c r="B38" s="5" t="s">
+        <v>728</v>
+      </c>
+      <c r="C38" s="14" t="s">
+        <v>723</v>
+      </c>
       <c r="D38" s="10" t="s">
         <v>726</v>
       </c>
       <c r="E38" s="7"/>
-      <c r="F38" s="10" t="s">
-        <v>737</v>
+      <c r="F38" s="10">
+        <v>-0.7</v>
       </c>
       <c r="G38" s="5" t="s">
-        <v>730</v>
+        <v>727</v>
       </c>
     </row>
     <row r="39">
@@ -25777,11 +25787,11 @@
       <c r="B39" s="6"/>
       <c r="C39" s="7"/>
       <c r="D39" s="10" t="s">
-        <v>740</v>
+        <v>741</v>
       </c>
       <c r="E39" s="7"/>
-      <c r="F39" s="10" t="s">
-        <v>737</v>
+      <c r="F39" s="10">
+        <v>-6.17</v>
       </c>
       <c r="G39" s="5" t="s">
         <v>727</v>
@@ -25792,15 +25802,21 @@
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"J.Jill, Inc. (NYSE:JILL)")</f>
         <v>J.Jill, Inc. (NYSE:JILL)</v>
       </c>
-      <c r="B40" s="6"/>
-      <c r="C40" s="7"/>
-      <c r="D40" s="7"/>
+      <c r="B40" s="5" t="s">
+        <v>728</v>
+      </c>
+      <c r="C40" s="14" t="s">
+        <v>723</v>
+      </c>
+      <c r="D40" s="10" t="s">
+        <v>736</v>
+      </c>
       <c r="E40" s="7"/>
       <c r="F40" s="10">
-        <v>7.78</v>
+        <v>6.35</v>
       </c>
       <c r="G40" s="5" t="s">
-        <v>734</v>
+        <v>748</v>
       </c>
     </row>
     <row r="41">
@@ -25810,9 +25826,13 @@
       </c>
       <c r="B41" s="6"/>
       <c r="C41" s="7"/>
-      <c r="D41" s="7"/>
+      <c r="D41" s="10" t="s">
+        <v>726</v>
+      </c>
       <c r="E41" s="7"/>
-      <c r="F41" s="7"/>
+      <c r="F41" s="10">
+        <v>30.94</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="6" t="str">
@@ -25821,9 +25841,13 @@
       </c>
       <c r="B42" s="6"/>
       <c r="C42" s="7"/>
-      <c r="D42" s="7"/>
+      <c r="D42" s="10" t="s">
+        <v>726</v>
+      </c>
       <c r="E42" s="7"/>
-      <c r="F42" s="7"/>
+      <c r="F42" s="10">
+        <v>12.54</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="6" t="str">
@@ -25832,9 +25856,13 @@
       </c>
       <c r="B43" s="6"/>
       <c r="C43" s="7"/>
-      <c r="D43" s="7"/>
+      <c r="D43" s="10" t="s">
+        <v>726</v>
+      </c>
       <c r="E43" s="7"/>
-      <c r="F43" s="7"/>
+      <c r="F43" s="10">
+        <v>18.01</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="6" t="str">
@@ -25843,9 +25871,13 @@
       </c>
       <c r="B44" s="6"/>
       <c r="C44" s="7"/>
-      <c r="D44" s="7"/>
+      <c r="D44" s="10" t="s">
+        <v>726</v>
+      </c>
       <c r="E44" s="7"/>
-      <c r="F44" s="7"/>
+      <c r="F44" s="10">
+        <v>13.31</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="6" t="str">
@@ -25854,9 +25886,13 @@
       </c>
       <c r="B45" s="6"/>
       <c r="C45" s="7"/>
-      <c r="D45" s="7"/>
+      <c r="D45" s="10" t="s">
+        <v>726</v>
+      </c>
       <c r="E45" s="7"/>
-      <c r="F45" s="7"/>
+      <c r="F45" s="10">
+        <v>24.58</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="6" t="str">
@@ -25865,9 +25901,13 @@
       </c>
       <c r="B46" s="6"/>
       <c r="C46" s="7"/>
-      <c r="D46" s="7"/>
+      <c r="D46" s="10" t="s">
+        <v>749</v>
+      </c>
       <c r="E46" s="7"/>
-      <c r="F46" s="7"/>
+      <c r="F46" s="10">
+        <v>66.65</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="6" t="str">
@@ -25876,9 +25916,13 @@
       </c>
       <c r="B47" s="6"/>
       <c r="C47" s="7"/>
-      <c r="D47" s="7"/>
+      <c r="D47" s="10" t="s">
+        <v>736</v>
+      </c>
       <c r="E47" s="7"/>
-      <c r="F47" s="7"/>
+      <c r="F47" s="10">
+        <v>-1.94</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="6" t="str">
@@ -25887,9 +25931,13 @@
       </c>
       <c r="B48" s="6"/>
       <c r="C48" s="7"/>
-      <c r="D48" s="7"/>
+      <c r="D48" s="10" t="s">
+        <v>726</v>
+      </c>
       <c r="E48" s="7"/>
-      <c r="F48" s="7"/>
+      <c r="F48" s="10">
+        <v>-377.0</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="6" t="str">
@@ -25898,9 +25946,13 @@
       </c>
       <c r="B49" s="6"/>
       <c r="C49" s="7"/>
-      <c r="D49" s="7"/>
+      <c r="D49" s="10" t="s">
+        <v>726</v>
+      </c>
       <c r="E49" s="7"/>
-      <c r="F49" s="7"/>
+      <c r="F49" s="10">
+        <v>137.73</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="6" t="str">
@@ -25909,9 +25961,13 @@
       </c>
       <c r="B50" s="6"/>
       <c r="C50" s="7"/>
-      <c r="D50" s="7"/>
+      <c r="D50" s="10" t="s">
+        <v>738</v>
+      </c>
       <c r="E50" s="7"/>
-      <c r="F50" s="7"/>
+      <c r="F50" s="10">
+        <v>-29.2</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="6" t="str">
@@ -25920,9 +25976,13 @@
       </c>
       <c r="B51" s="6"/>
       <c r="C51" s="7"/>
-      <c r="D51" s="7"/>
+      <c r="D51" s="10" t="s">
+        <v>741</v>
+      </c>
       <c r="E51" s="7"/>
-      <c r="F51" s="7"/>
+      <c r="F51" s="10">
+        <v>-6.18</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="6" t="str">
@@ -25931,9 +25991,13 @@
       </c>
       <c r="B52" s="6"/>
       <c r="C52" s="7"/>
-      <c r="D52" s="7"/>
+      <c r="D52" s="10" t="s">
+        <v>731</v>
+      </c>
       <c r="E52" s="7"/>
-      <c r="F52" s="7"/>
+      <c r="F52" s="10">
+        <v>-6.7</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="6" t="str">
@@ -25942,9 +26006,13 @@
       </c>
       <c r="B53" s="6"/>
       <c r="C53" s="7"/>
-      <c r="D53" s="7"/>
+      <c r="D53" s="10" t="s">
+        <v>736</v>
+      </c>
       <c r="E53" s="7"/>
-      <c r="F53" s="7"/>
+      <c r="F53" s="10">
+        <v>12.1</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="6" t="str">
@@ -25953,9 +26021,13 @@
       </c>
       <c r="B54" s="6"/>
       <c r="C54" s="7"/>
-      <c r="D54" s="7"/>
+      <c r="D54" s="10" t="s">
+        <v>724</v>
+      </c>
       <c r="E54" s="7"/>
-      <c r="F54" s="7"/>
+      <c r="F54" s="10">
+        <v>-20.9</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="6" t="str">
@@ -25964,9 +26036,13 @@
       </c>
       <c r="B55" s="6"/>
       <c r="C55" s="7"/>
-      <c r="D55" s="7"/>
+      <c r="D55" s="10" t="s">
+        <v>736</v>
+      </c>
       <c r="E55" s="7"/>
-      <c r="F55" s="7"/>
+      <c r="F55" s="10">
+        <v>-10.55</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="6" t="str">
@@ -25975,9 +26051,13 @@
       </c>
       <c r="B56" s="6"/>
       <c r="C56" s="7"/>
-      <c r="D56" s="7"/>
+      <c r="D56" s="10" t="s">
+        <v>741</v>
+      </c>
       <c r="E56" s="7"/>
-      <c r="F56" s="7"/>
+      <c r="F56" s="10">
+        <v>-0.14</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="6" t="str">
@@ -25986,9 +26066,13 @@
       </c>
       <c r="B57" s="6"/>
       <c r="C57" s="7"/>
-      <c r="D57" s="7"/>
+      <c r="D57" s="10" t="s">
+        <v>741</v>
+      </c>
       <c r="E57" s="7"/>
-      <c r="F57" s="7"/>
+      <c r="F57" s="10">
+        <v>-5.24</v>
+      </c>
     </row>
     <row r="58">
       <c r="B58" s="6"/>
@@ -32608,7 +32692,9 @@
     <hyperlink r:id="rId9" ref="C10"/>
     <hyperlink r:id="rId10" ref="C11"/>
     <hyperlink r:id="rId11" ref="C35"/>
+    <hyperlink r:id="rId12" ref="C38"/>
+    <hyperlink r:id="rId13" ref="C40"/>
   </hyperlinks>
-  <drawing r:id="rId12"/>
+  <drawing r:id="rId14"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update Hamilton Beach qualitative assessment
</commit_message>
<xml_diff>
--- a/public/research/initial-screenings/Initial Screening (Under 1B MC, Over $0 NI).xlsx
+++ b/public/research/initial-screenings/Initial Screening (Under 1B MC, Over $0 NI).xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2023" uniqueCount="750">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2025" uniqueCount="750">
   <si>
     <t>Entity Name</t>
   </si>
@@ -25726,8 +25726,12 @@
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Hamilton Beach Brands Holding Company (NYSE:HBB)")</f>
         <v>Hamilton Beach Brands Holding Company (NYSE:HBB)</v>
       </c>
-      <c r="B36" s="6"/>
-      <c r="C36" s="7"/>
+      <c r="B36" s="5" t="s">
+        <v>728</v>
+      </c>
+      <c r="C36" s="14" t="s">
+        <v>723</v>
+      </c>
       <c r="D36" s="10" t="s">
         <v>726</v>
       </c>
@@ -32692,9 +32696,10 @@
     <hyperlink r:id="rId9" ref="C10"/>
     <hyperlink r:id="rId10" ref="C11"/>
     <hyperlink r:id="rId11" ref="C35"/>
-    <hyperlink r:id="rId12" ref="C38"/>
-    <hyperlink r:id="rId13" ref="C40"/>
+    <hyperlink r:id="rId12" ref="C36"/>
+    <hyperlink r:id="rId13" ref="C38"/>
+    <hyperlink r:id="rId14" ref="C40"/>
   </hyperlinks>
-  <drawing r:id="rId14"/>
+  <drawing r:id="rId15"/>
 </worksheet>
 </file>
</xml_diff>